<commit_message>
ATD pipeline, rename HARA parameters
</commit_message>
<xml_diff>
--- a/service/analyse/Automotive-threat-database.xlsx
+++ b/service/analyse/Automotive-threat-database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nalin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://epitafr-my.sharepoint.com/personal/khaoula_sghaier_epita_fr/Documents/Bureau/PhD_Khaoula/Code/Risk_assessment/RiskAssessment/service/analyse/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{756F44AD-4C1B-4EA5-922E-98860B3C5851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{756F44AD-4C1B-4EA5-922E-98860B3C5851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E335EE13-48E3-4E85-9C51-5FA19BDCA113}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9D3130C4-4E28-4A4B-8AD1-48FB110EC596}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9D3130C4-4E28-4A4B-8AD1-48FB110EC596}"/>
   </bookViews>
   <sheets>
     <sheet name="ATD" sheetId="1" r:id="rId1"/>
@@ -9716,10 +9716,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -9727,26 +9726,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="34">
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -9910,6 +9890,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -10057,46 +10047,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16E9BB53-937D-4023-A88B-D3B4B37A36B9}" name="Table2" displayName="Table2" ref="A1:AF510" totalsRowCount="1" headerRowDxfId="34" dataDxfId="33" totalsRowDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{16E9BB53-937D-4023-A88B-D3B4B37A36B9}" name="Table2" displayName="Table2" ref="A1:AF510" totalsRowCount="1" headerRowDxfId="33" dataDxfId="32" totalsRowDxfId="31">
   <autoFilter ref="A1:AF509" xr:uid="{16E9BB53-937D-4023-A88B-D3B4B37A36B9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AF509">
     <sortCondition ref="B1:B509"/>
   </sortState>
   <tableColumns count="32">
-    <tableColumn id="36" xr3:uid="{69733A95-AF07-44B1-A3CE-EFD40CF920F9}" name="ATD_ID2" totalsRowDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{79AF4B85-91F5-413A-939C-C498BDEC714D}" name="Index" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{03F330A7-3E95-47C0-ABD8-6A01AB5AA9D6}" name="Unique_ID" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{37D6008C-19D1-41E8-931C-DE096DD7645C}" name="CVE_ID" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{5106A034-84C4-4462-B659-37D950B4E9C1}" name="AAD_ID" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{38A0432C-E0B2-4FAC-9624-37C480BD6E8C}" name="AAD_Single_ID" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{3F2DF04A-81D0-41FD-8514-872FA09CAA13}" name="Description" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{A0CBF2E0-5382-43C6-BEF3-128BC4D9B94B}" name="Reference" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{FF3EC133-D037-4B3B-8667-119B6E32F363}" name="Published_year" dataDxfId="24"/>
-    <tableColumn id="16" xr3:uid="{63B38153-AC51-4B8A-AC94-D424CFDBB456}" name="Safety" dataDxfId="5"/>
-    <tableColumn id="17" xr3:uid="{69F2112D-2A52-4056-9455-108F3AEDF8F3}" name="Financial" dataDxfId="4"/>
-    <tableColumn id="18" xr3:uid="{1927783A-5092-4DE2-A4B4-D69985E4C7DB}" name="Operational" dataDxfId="3"/>
-    <tableColumn id="19" xr3:uid="{F735F343-D662-4FDA-8180-2A2349C67017}" name="Privacy" dataDxfId="2"/>
-    <tableColumn id="26" xr3:uid="{7816C86D-43FF-43B4-B114-5D1E4D12CF31}" name="Systemic" totalsRowFunction="count" dataDxfId="1">
+    <tableColumn id="36" xr3:uid="{69733A95-AF07-44B1-A3CE-EFD40CF920F9}" name="ATD_ID2"/>
+    <tableColumn id="2" xr3:uid="{79AF4B85-91F5-413A-939C-C498BDEC714D}" name="Index" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{03F330A7-3E95-47C0-ABD8-6A01AB5AA9D6}" name="Unique_ID" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{37D6008C-19D1-41E8-931C-DE096DD7645C}" name="CVE_ID" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{5106A034-84C4-4462-B659-37D950B4E9C1}" name="AAD_ID" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{38A0432C-E0B2-4FAC-9624-37C480BD6E8C}" name="AAD_Single_ID" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{3F2DF04A-81D0-41FD-8514-872FA09CAA13}" name="Description" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{A0CBF2E0-5382-43C6-BEF3-128BC4D9B94B}" name="Reference" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{FF3EC133-D037-4B3B-8667-119B6E32F363}" name="Published_year" dataDxfId="23"/>
+    <tableColumn id="16" xr3:uid="{63B38153-AC51-4B8A-AC94-D424CFDBB456}" name="Safety" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{69F2112D-2A52-4056-9455-108F3AEDF8F3}" name="Financial" dataDxfId="21"/>
+    <tableColumn id="18" xr3:uid="{1927783A-5092-4DE2-A4B4-D69985E4C7DB}" name="Operational" dataDxfId="20"/>
+    <tableColumn id="19" xr3:uid="{F735F343-D662-4FDA-8180-2A2349C67017}" name="Privacy" dataDxfId="19"/>
+    <tableColumn id="26" xr3:uid="{7816C86D-43FF-43B4-B114-5D1E4D12CF31}" name="Systemic" totalsRowFunction="count" dataDxfId="18">
       <calculatedColumnFormula>IF(AND(OR(T2="A", T2="N"), J2="Yes"), "Potentially Systemic", "Not Systemic")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{5290E860-233E-41D1-A6E4-7CCE24F5A0B9}" name="CWE_ID" dataDxfId="23"/>
-    <tableColumn id="11" xr3:uid="{B5C22FD3-196A-4430-B29A-95430005532C}" name="CVSS3.x_vector_string" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{5FFAFDDD-B908-4BF9-9ACD-1102163466C4}" name="3_Base_score" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{A2AD1760-3488-42E0-938E-C8A83614E919}" name="3_Exploitability_score" dataDxfId="20"/>
-    <tableColumn id="14" xr3:uid="{B59CEE9C-ED3E-4FC1-89EE-FC9017BA1D04}" name="3_Impact_score" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{7216E6B6-0C61-4EE9-9F56-5E2449C24E4D}" name="Attack_vector" dataDxfId="18"/>
-    <tableColumn id="20" xr3:uid="{ACAC3EE5-63DE-488E-9EC7-2E2AAFDF2BD3}" name="CVSS_2.0_vector_string" dataDxfId="17"/>
-    <tableColumn id="21" xr3:uid="{3A47EF21-C0BA-46E7-9723-362D4BCDA1C8}" name="2_Base_score" dataDxfId="16"/>
-    <tableColumn id="22" xr3:uid="{ED4D82AB-FDB2-46FC-9170-1065F47AAAAE}" name="2_Exploitability_score" dataDxfId="15"/>
-    <tableColumn id="23" xr3:uid="{EE3B47EA-612D-4142-9D07-635B0894957D}" name="2_Impact_score" dataDxfId="14"/>
-    <tableColumn id="24" xr3:uid="{434EA9E4-BF0A-489F-99A8-94DEBD00713A}" name="Database" dataDxfId="13"/>
-    <tableColumn id="25" xr3:uid="{BBA07B46-4BC6-41D8-A60D-6510B4E2109E}" name="CVE_ID_other" dataDxfId="12"/>
-    <tableColumn id="27" xr3:uid="{4F21D6C0-0CEC-4639-B3BF-9349E760DDF7}" name="Attack Base" dataDxfId="11"/>
-    <tableColumn id="28" xr3:uid="{48C5FC19-2AD2-49F0-ABC6-A9A01BD5B13C}" name="Attack Type" dataDxfId="10"/>
-    <tableColumn id="29" xr3:uid="{CC2C2775-0306-4E07-9C3A-5CC0E10091BB}" name="Violated Security Property" dataDxfId="9"/>
-    <tableColumn id="30" xr3:uid="{0AA4407A-C16C-41A0-919D-A00BBD5C6877}" name="Interface" dataDxfId="8"/>
-    <tableColumn id="31" xr3:uid="{FE7B0E48-C793-4DB4-AD78-25E7964BCD65}" name="Consequence" dataDxfId="7"/>
-    <tableColumn id="32" xr3:uid="{F2E5F5E3-0324-47E1-B04A-E3ED34FB7DB4}" name="Component" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{5290E860-233E-41D1-A6E4-7CCE24F5A0B9}" name="CWE_ID" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{B5C22FD3-196A-4430-B29A-95430005532C}" name="CVSS3.x_vector_string" dataDxfId="16"/>
+    <tableColumn id="12" xr3:uid="{5FFAFDDD-B908-4BF9-9ACD-1102163466C4}" name="3_Base_score" dataDxfId="15"/>
+    <tableColumn id="13" xr3:uid="{A2AD1760-3488-42E0-938E-C8A83614E919}" name="3_Exploitability_score" dataDxfId="14"/>
+    <tableColumn id="14" xr3:uid="{B59CEE9C-ED3E-4FC1-89EE-FC9017BA1D04}" name="3_Impact_score" dataDxfId="13"/>
+    <tableColumn id="15" xr3:uid="{7216E6B6-0C61-4EE9-9F56-5E2449C24E4D}" name="Attack_vector" dataDxfId="12"/>
+    <tableColumn id="20" xr3:uid="{ACAC3EE5-63DE-488E-9EC7-2E2AAFDF2BD3}" name="CVSS_2.0_vector_string" dataDxfId="11"/>
+    <tableColumn id="21" xr3:uid="{3A47EF21-C0BA-46E7-9723-362D4BCDA1C8}" name="2_Base_score" dataDxfId="10"/>
+    <tableColumn id="22" xr3:uid="{ED4D82AB-FDB2-46FC-9170-1065F47AAAAE}" name="2_Exploitability_score" dataDxfId="9"/>
+    <tableColumn id="23" xr3:uid="{EE3B47EA-612D-4142-9D07-635B0894957D}" name="2_Impact_score" dataDxfId="8"/>
+    <tableColumn id="24" xr3:uid="{434EA9E4-BF0A-489F-99A8-94DEBD00713A}" name="Database" dataDxfId="7"/>
+    <tableColumn id="25" xr3:uid="{BBA07B46-4BC6-41D8-A60D-6510B4E2109E}" name="CVE_ID_other" dataDxfId="6"/>
+    <tableColumn id="27" xr3:uid="{4F21D6C0-0CEC-4639-B3BF-9349E760DDF7}" name="Attack Base" dataDxfId="5"/>
+    <tableColumn id="28" xr3:uid="{48C5FC19-2AD2-49F0-ABC6-A9A01BD5B13C}" name="Attack Type" dataDxfId="4"/>
+    <tableColumn id="29" xr3:uid="{CC2C2775-0306-4E07-9C3A-5CC0E10091BB}" name="Violated Security Property" dataDxfId="3"/>
+    <tableColumn id="30" xr3:uid="{0AA4407A-C16C-41A0-919D-A00BBD5C6877}" name="Interface" dataDxfId="2"/>
+    <tableColumn id="31" xr3:uid="{FE7B0E48-C793-4DB4-AD78-25E7964BCD65}" name="Consequence" dataDxfId="1"/>
+    <tableColumn id="32" xr3:uid="{F2E5F5E3-0324-47E1-B04A-E3ED34FB7DB4}" name="Component" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10482,19 +10472,19 @@
       <c r="I1" t="s">
         <v>2688</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>2681</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>2680</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>2679</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>2678</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="3" t="s">
         <v>2696</v>
       </c>
       <c r="O1" t="s">
@@ -10584,7 +10574,7 @@
         <v>43</v>
       </c>
       <c r="N2" t="str">
-        <f>IF(AND(OR(T2="A", T2="N"), J2="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N2:N65" si="0">IF(AND(OR(T2="A", T2="N"), J2="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Potentially Systemic</v>
       </c>
       <c r="O2" t="s">
@@ -10644,7 +10634,7 @@
         <v>43</v>
       </c>
       <c r="N3" t="str">
-        <f>IF(AND(OR(T3="A", T3="N"), J3="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O3" t="s">
@@ -10710,7 +10700,7 @@
         <v>43</v>
       </c>
       <c r="N4" t="str">
-        <f>IF(AND(OR(T4="A", T4="N"), J4="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O4" t="s">
@@ -10764,7 +10754,7 @@
         <v>43</v>
       </c>
       <c r="N5" t="str">
-        <f>IF(AND(OR(T5="A", T5="N"), J5="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O5" t="s">
@@ -10821,7 +10811,7 @@
         <v>43</v>
       </c>
       <c r="N6" t="str">
-        <f>IF(AND(OR(T6="A", T6="N"), J6="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O6" t="s">
@@ -10887,7 +10877,7 @@
         <v>43</v>
       </c>
       <c r="N7" t="str">
-        <f>IF(AND(OR(T7="A", T7="N"), J7="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O7" t="s">
@@ -10950,7 +10940,7 @@
         <v>43</v>
       </c>
       <c r="N8" t="str">
-        <f>IF(AND(OR(T8="A", T8="N"), J8="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O8" t="s">
@@ -11013,7 +11003,7 @@
         <v>43</v>
       </c>
       <c r="N9" t="str">
-        <f>IF(AND(OR(T9="A", T9="N"), J9="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O9" t="s">
@@ -11079,7 +11069,7 @@
         <v>43</v>
       </c>
       <c r="N10" t="str">
-        <f>IF(AND(OR(T10="A", T10="N"), J10="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O10" t="s">
@@ -11148,7 +11138,7 @@
         <v>43</v>
       </c>
       <c r="N11" t="str">
-        <f>IF(AND(OR(T11="A", T11="N"), J11="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O11" t="s">
@@ -11220,7 +11210,7 @@
         <v>43</v>
       </c>
       <c r="N12" t="str">
-        <f>IF(AND(OR(T12="A", T12="N"), J12="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O12" t="s">
@@ -11280,7 +11270,7 @@
         <v>43</v>
       </c>
       <c r="N13" t="str">
-        <f>IF(AND(OR(T13="A", T13="N"), J13="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O13" t="s">
@@ -11340,7 +11330,7 @@
         <v>43</v>
       </c>
       <c r="N14" t="str">
-        <f>IF(AND(OR(T14="A", T14="N"), J14="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O14" t="s">
@@ -11400,7 +11390,7 @@
         <v>43</v>
       </c>
       <c r="N15" t="str">
-        <f>IF(AND(OR(T15="A", T15="N"), J15="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O15" t="s">
@@ -11451,7 +11441,7 @@
         <v>43</v>
       </c>
       <c r="N16" t="str">
-        <f>IF(AND(OR(T16="A", T16="N"), J16="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O16" t="s">
@@ -11505,7 +11495,7 @@
         <v>43</v>
       </c>
       <c r="N17" t="str">
-        <f>IF(AND(OR(T17="A", T17="N"), J17="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O17" t="s">
@@ -11556,7 +11546,7 @@
         <v>43</v>
       </c>
       <c r="N18" t="str">
-        <f>IF(AND(OR(T18="A", T18="N"), J18="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O18" t="s">
@@ -11607,7 +11597,7 @@
         <v>43</v>
       </c>
       <c r="N19" t="str">
-        <f>IF(AND(OR(T19="A", T19="N"), J19="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O19" t="s">
@@ -11664,7 +11654,7 @@
         <v>43</v>
       </c>
       <c r="N20" t="str">
-        <f>IF(AND(OR(T20="A", T20="N"), J20="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O20" t="s">
@@ -11721,7 +11711,7 @@
         <v>43</v>
       </c>
       <c r="N21" t="str">
-        <f>IF(AND(OR(T21="A", T21="N"), J21="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O21" t="s">
@@ -11772,7 +11762,7 @@
         <v>43</v>
       </c>
       <c r="N22" t="str">
-        <f>IF(AND(OR(T22="A", T22="N"), J22="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O22" t="s">
@@ -11829,7 +11819,7 @@
         <v>43</v>
       </c>
       <c r="N23" t="str">
-        <f>IF(AND(OR(T23="A", T23="N"), J23="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O23" t="s">
@@ -11898,7 +11888,7 @@
         <v>43</v>
       </c>
       <c r="N24" t="str">
-        <f>IF(AND(OR(T24="A", T24="N"), J24="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O24" t="s">
@@ -11967,7 +11957,7 @@
         <v>43</v>
       </c>
       <c r="N25" t="str">
-        <f>IF(AND(OR(T25="A", T25="N"), J25="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O25" t="s">
@@ -12036,7 +12026,7 @@
         <v>43</v>
       </c>
       <c r="N26" t="str">
-        <f>IF(AND(OR(T26="A", T26="N"), J26="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O26" t="s">
@@ -12105,7 +12095,7 @@
         <v>43</v>
       </c>
       <c r="N27" t="str">
-        <f>IF(AND(OR(T27="A", T27="N"), J27="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O27" t="s">
@@ -12174,7 +12164,7 @@
         <v>43</v>
       </c>
       <c r="N28" t="str">
-        <f>IF(AND(OR(T28="A", T28="N"), J28="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O28" t="s">
@@ -12243,7 +12233,7 @@
         <v>43</v>
       </c>
       <c r="N29" t="str">
-        <f>IF(AND(OR(T29="A", T29="N"), J29="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O29" t="s">
@@ -12312,7 +12302,7 @@
         <v>43</v>
       </c>
       <c r="N30" t="str">
-        <f>IF(AND(OR(T30="A", T30="N"), J30="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O30" t="s">
@@ -12381,7 +12371,7 @@
         <v>43</v>
       </c>
       <c r="N31" t="str">
-        <f>IF(AND(OR(T31="A", T31="N"), J31="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O31" t="s">
@@ -12453,7 +12443,7 @@
         <v>43</v>
       </c>
       <c r="N32" t="str">
-        <f>IF(AND(OR(T32="A", T32="N"), J32="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O32" t="s">
@@ -12519,7 +12509,7 @@
         <v>43</v>
       </c>
       <c r="N33" t="str">
-        <f>IF(AND(OR(T33="A", T33="N"), J33="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O33" t="s">
@@ -12573,7 +12563,7 @@
         <v>43</v>
       </c>
       <c r="N34" t="str">
-        <f>IF(AND(OR(T34="A", T34="N"), J34="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O34" t="s">
@@ -12627,7 +12617,7 @@
         <v>43</v>
       </c>
       <c r="N35" t="str">
-        <f>IF(AND(OR(T35="A", T35="N"), J35="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O35" t="s">
@@ -12681,7 +12671,7 @@
         <v>43</v>
       </c>
       <c r="N36" t="str">
-        <f>IF(AND(OR(T36="A", T36="N"), J36="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O36" t="s">
@@ -12738,7 +12728,7 @@
         <v>43</v>
       </c>
       <c r="N37" t="str">
-        <f>IF(AND(OR(T37="A", T37="N"), J37="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O37" t="s">
@@ -12798,7 +12788,7 @@
         <v>43</v>
       </c>
       <c r="N38" t="str">
-        <f>IF(AND(OR(T38="A", T38="N"), J38="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="P38" t="s">
@@ -12849,7 +12839,7 @@
         <v>43</v>
       </c>
       <c r="N39" t="str">
-        <f>IF(AND(OR(T39="A", T39="N"), J39="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="P39" t="s">
@@ -12900,7 +12890,7 @@
         <v>43</v>
       </c>
       <c r="N40" t="str">
-        <f>IF(AND(OR(T40="A", T40="N"), J40="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O40" t="s">
@@ -12951,7 +12941,7 @@
         <v>43</v>
       </c>
       <c r="N41" t="str">
-        <f>IF(AND(OR(T41="A", T41="N"), J41="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O41" t="s">
@@ -13011,7 +13001,7 @@
         <v>43</v>
       </c>
       <c r="N42" t="str">
-        <f>IF(AND(OR(T42="A", T42="N"), J42="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O42" t="s">
@@ -13065,7 +13055,7 @@
         <v>43</v>
       </c>
       <c r="N43" t="str">
-        <f>IF(AND(OR(T43="A", T43="N"), J43="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="P43" t="s">
@@ -13119,7 +13109,7 @@
         <v>43</v>
       </c>
       <c r="N44" t="str">
-        <f>IF(AND(OR(T44="A", T44="N"), J44="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O44" t="s">
@@ -13176,7 +13166,7 @@
         <v>43</v>
       </c>
       <c r="N45" t="str">
-        <f>IF(AND(OR(T45="A", T45="N"), J45="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O45" t="s">
@@ -13236,7 +13226,7 @@
         <v>43</v>
       </c>
       <c r="N46" t="str">
-        <f>IF(AND(OR(T46="A", T46="N"), J46="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O46" t="s">
@@ -13293,7 +13283,7 @@
         <v>43</v>
       </c>
       <c r="N47" t="str">
-        <f>IF(AND(OR(T47="A", T47="N"), J47="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O47" t="s">
@@ -13344,7 +13334,7 @@
         <v>43</v>
       </c>
       <c r="N48" t="str">
-        <f>IF(AND(OR(T48="A", T48="N"), J48="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O48" t="s">
@@ -13401,7 +13391,7 @@
         <v>43</v>
       </c>
       <c r="N49" t="str">
-        <f>IF(AND(OR(T49="A", T49="N"), J49="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O49" t="s">
@@ -13458,7 +13448,7 @@
         <v>43</v>
       </c>
       <c r="N50" t="str">
-        <f>IF(AND(OR(T50="A", T50="N"), J50="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O50" t="s">
@@ -13518,7 +13508,7 @@
         <v>43</v>
       </c>
       <c r="N51" t="str">
-        <f>IF(AND(OR(T51="A", T51="N"), J51="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O51" t="s">
@@ -13572,7 +13562,7 @@
         <v>43</v>
       </c>
       <c r="N52" t="str">
-        <f>IF(AND(OR(T52="A", T52="N"), J52="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O52" t="s">
@@ -13635,7 +13625,7 @@
         <v>43</v>
       </c>
       <c r="N53" t="str">
-        <f>IF(AND(OR(T53="A", T53="N"), J53="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O53" t="s">
@@ -13698,7 +13688,7 @@
         <v>43</v>
       </c>
       <c r="N54" t="str">
-        <f>IF(AND(OR(T54="A", T54="N"), J54="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O54" t="s">
@@ -13770,7 +13760,7 @@
         <v>43</v>
       </c>
       <c r="N55" t="str">
-        <f>IF(AND(OR(T55="A", T55="N"), J55="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O55" t="s">
@@ -13833,7 +13823,7 @@
         <v>43</v>
       </c>
       <c r="N56" t="str">
-        <f>IF(AND(OR(T56="A", T56="N"), J56="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O56" t="s">
@@ -13896,7 +13886,7 @@
         <v>43</v>
       </c>
       <c r="N57" t="str">
-        <f>IF(AND(OR(T57="A", T57="N"), J57="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O57" t="s">
@@ -13962,7 +13952,7 @@
         <v>43</v>
       </c>
       <c r="N58" t="str">
-        <f>IF(AND(OR(T58="A", T58="N"), J58="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O58" t="s">
@@ -14025,7 +14015,7 @@
         <v>43</v>
       </c>
       <c r="N59" t="str">
-        <f>IF(AND(OR(T59="A", T59="N"), J59="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O59" t="s">
@@ -14088,7 +14078,7 @@
         <v>43</v>
       </c>
       <c r="N60" t="str">
-        <f>IF(AND(OR(T60="A", T60="N"), J60="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O60" t="s">
@@ -14154,7 +14144,7 @@
         <v>43</v>
       </c>
       <c r="N61" t="str">
-        <f>IF(AND(OR(T61="A", T61="N"), J61="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O61" t="s">
@@ -14220,7 +14210,7 @@
         <v>43</v>
       </c>
       <c r="N62" t="str">
-        <f>IF(AND(OR(T62="A", T62="N"), J62="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O62" t="s">
@@ -14286,7 +14276,7 @@
         <v>43</v>
       </c>
       <c r="N63" t="str">
-        <f>IF(AND(OR(T63="A", T63="N"), J63="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O63" t="s">
@@ -14352,7 +14342,7 @@
         <v>43</v>
       </c>
       <c r="N64" t="str">
-        <f>IF(AND(OR(T64="A", T64="N"), J64="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O64" t="s">
@@ -14421,7 +14411,7 @@
         <v>43</v>
       </c>
       <c r="N65" t="str">
-        <f>IF(AND(OR(T65="A", T65="N"), J65="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="0"/>
         <v>Not Systemic</v>
       </c>
       <c r="O65" t="s">
@@ -14484,7 +14474,7 @@
         <v>43</v>
       </c>
       <c r="N66" t="str">
-        <f>IF(AND(OR(T66="A", T66="N"), J66="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N66:N129" si="1">IF(AND(OR(T66="A", T66="N"), J66="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O66" t="s">
@@ -14553,7 +14543,7 @@
         <v>43</v>
       </c>
       <c r="N67" t="str">
-        <f>IF(AND(OR(T67="A", T67="N"), J67="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O67" t="s">
@@ -14625,7 +14615,7 @@
         <v>43</v>
       </c>
       <c r="N68" t="str">
-        <f>IF(AND(OR(T68="A", T68="N"), J68="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O68" t="s">
@@ -14694,7 +14684,7 @@
         <v>43</v>
       </c>
       <c r="N69" t="str">
-        <f>IF(AND(OR(T69="A", T69="N"), J69="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O69" t="s">
@@ -14763,7 +14753,7 @@
         <v>43</v>
       </c>
       <c r="N70" t="str">
-        <f>IF(AND(OR(T70="A", T70="N"), J70="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O70" t="s">
@@ -14829,7 +14819,7 @@
         <v>43</v>
       </c>
       <c r="N71" t="str">
-        <f>IF(AND(OR(T71="A", T71="N"), J71="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O71" t="s">
@@ -14895,7 +14885,7 @@
         <v>43</v>
       </c>
       <c r="N72" t="str">
-        <f>IF(AND(OR(T72="A", T72="N"), J72="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O72" t="s">
@@ -14961,7 +14951,7 @@
         <v>43</v>
       </c>
       <c r="N73" t="str">
-        <f>IF(AND(OR(T73="A", T73="N"), J73="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O73" t="s">
@@ -15027,7 +15017,7 @@
         <v>43</v>
       </c>
       <c r="N74" t="str">
-        <f>IF(AND(OR(T74="A", T74="N"), J74="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O74" t="s">
@@ -15093,7 +15083,7 @@
         <v>43</v>
       </c>
       <c r="N75" t="str">
-        <f>IF(AND(OR(T75="A", T75="N"), J75="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O75" t="s">
@@ -15156,7 +15146,7 @@
         <v>43</v>
       </c>
       <c r="N76" t="str">
-        <f>IF(AND(OR(T76="A", T76="N"), J76="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O76" t="s">
@@ -15219,7 +15209,7 @@
         <v>43</v>
       </c>
       <c r="N77" t="str">
-        <f>IF(AND(OR(T77="A", T77="N"), J77="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O77" t="s">
@@ -15270,7 +15260,7 @@
         <v>43</v>
       </c>
       <c r="N78" t="str">
-        <f>IF(AND(OR(T78="A", T78="N"), J78="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O78" t="s">
@@ -15342,7 +15332,7 @@
         <v>43</v>
       </c>
       <c r="N79" t="str">
-        <f>IF(AND(OR(T79="A", T79="N"), J79="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O79" t="s">
@@ -15414,7 +15404,7 @@
         <v>43</v>
       </c>
       <c r="N80" t="str">
-        <f>IF(AND(OR(T80="A", T80="N"), J80="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O80" t="s">
@@ -15465,7 +15455,7 @@
         <v>43</v>
       </c>
       <c r="N81" t="str">
-        <f>IF(AND(OR(T81="A", T81="N"), J81="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O81" t="s">
@@ -15534,7 +15524,7 @@
         <v>43</v>
       </c>
       <c r="N82" t="str">
-        <f>IF(AND(OR(T82="A", T82="N"), J82="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O82" t="s">
@@ -15597,7 +15587,7 @@
         <v>43</v>
       </c>
       <c r="N83" t="str">
-        <f>IF(AND(OR(T83="A", T83="N"), J83="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O83" t="s">
@@ -15669,7 +15659,7 @@
         <v>43</v>
       </c>
       <c r="N84" t="str">
-        <f>IF(AND(OR(T84="A", T84="N"), J84="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O84" t="s">
@@ -15720,7 +15710,7 @@
         <v>43</v>
       </c>
       <c r="N85" t="str">
-        <f>IF(AND(OR(T85="A", T85="N"), J85="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O85" t="s">
@@ -15771,7 +15761,7 @@
         <v>43</v>
       </c>
       <c r="N86" t="str">
-        <f>IF(AND(OR(T86="A", T86="N"), J86="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O86" t="s">
@@ -15822,7 +15812,7 @@
         <v>43</v>
       </c>
       <c r="N87" t="str">
-        <f>IF(AND(OR(T87="A", T87="N"), J87="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O87" t="s">
@@ -15873,7 +15863,7 @@
         <v>43</v>
       </c>
       <c r="N88" t="str">
-        <f>IF(AND(OR(T88="A", T88="N"), J88="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O88" t="s">
@@ -15924,7 +15914,7 @@
         <v>43</v>
       </c>
       <c r="N89" t="str">
-        <f>IF(AND(OR(T89="A", T89="N"), J89="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O89" t="s">
@@ -15975,7 +15965,7 @@
         <v>43</v>
       </c>
       <c r="N90" t="str">
-        <f>IF(AND(OR(T90="A", T90="N"), J90="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O90" t="s">
@@ -16026,7 +16016,7 @@
         <v>43</v>
       </c>
       <c r="N91" t="str">
-        <f>IF(AND(OR(T91="A", T91="N"), J91="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O91" t="s">
@@ -16077,7 +16067,7 @@
         <v>43</v>
       </c>
       <c r="N92" t="str">
-        <f>IF(AND(OR(T92="A", T92="N"), J92="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O92" t="s">
@@ -16128,7 +16118,7 @@
         <v>43</v>
       </c>
       <c r="N93" t="str">
-        <f>IF(AND(OR(T93="A", T93="N"), J93="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O93" t="s">
@@ -16179,7 +16169,7 @@
         <v>43</v>
       </c>
       <c r="N94" t="str">
-        <f>IF(AND(OR(T94="A", T94="N"), J94="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O94" t="s">
@@ -16230,7 +16220,7 @@
         <v>43</v>
       </c>
       <c r="N95" t="str">
-        <f>IF(AND(OR(T95="A", T95="N"), J95="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O95" t="s">
@@ -16290,7 +16280,7 @@
         <v>43</v>
       </c>
       <c r="N96" t="str">
-        <f>IF(AND(OR(T96="A", T96="N"), J96="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O96" t="s">
@@ -16350,7 +16340,7 @@
         <v>43</v>
       </c>
       <c r="N97" t="str">
-        <f>IF(AND(OR(T97="A", T97="N"), J97="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O97" t="s">
@@ -16401,7 +16391,7 @@
         <v>43</v>
       </c>
       <c r="N98" t="str">
-        <f>IF(AND(OR(T98="A", T98="N"), J98="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O98" t="s">
@@ -16458,7 +16448,7 @@
         <v>43</v>
       </c>
       <c r="N99" t="str">
-        <f>IF(AND(OR(T99="A", T99="N"), J99="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O99" t="s">
@@ -16515,7 +16505,7 @@
         <v>43</v>
       </c>
       <c r="N100" t="str">
-        <f>IF(AND(OR(T100="A", T100="N"), J100="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O100" t="s">
@@ -16572,7 +16562,7 @@
         <v>43</v>
       </c>
       <c r="N101" t="str">
-        <f>IF(AND(OR(T101="A", T101="N"), J101="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O101" t="s">
@@ -16629,7 +16619,7 @@
         <v>43</v>
       </c>
       <c r="N102" t="str">
-        <f>IF(AND(OR(T102="A", T102="N"), J102="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O102" t="s">
@@ -16686,7 +16676,7 @@
         <v>43</v>
       </c>
       <c r="N103" t="str">
-        <f>IF(AND(OR(T103="A", T103="N"), J103="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O103" t="s">
@@ -16743,7 +16733,7 @@
         <v>43</v>
       </c>
       <c r="N104" t="str">
-        <f>IF(AND(OR(T104="A", T104="N"), J104="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O104" t="s">
@@ -16800,7 +16790,7 @@
         <v>43</v>
       </c>
       <c r="N105" t="str">
-        <f>IF(AND(OR(T105="A", T105="N"), J105="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O105" t="s">
@@ -16857,7 +16847,7 @@
         <v>43</v>
       </c>
       <c r="N106" t="str">
-        <f>IF(AND(OR(T106="A", T106="N"), J106="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O106" t="s">
@@ -16914,7 +16904,7 @@
         <v>43</v>
       </c>
       <c r="N107" t="str">
-        <f>IF(AND(OR(T107="A", T107="N"), J107="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O107" t="s">
@@ -16971,7 +16961,7 @@
         <v>43</v>
       </c>
       <c r="N108" t="str">
-        <f>IF(AND(OR(T108="A", T108="N"), J108="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O108" t="s">
@@ -17022,7 +17012,7 @@
         <v>43</v>
       </c>
       <c r="N109" t="str">
-        <f>IF(AND(OR(T109="A", T109="N"), J109="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O109" t="s">
@@ -17076,7 +17066,7 @@
         <v>43</v>
       </c>
       <c r="N110" t="str">
-        <f>IF(AND(OR(T110="A", T110="N"), J110="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O110" t="s">
@@ -17130,7 +17120,7 @@
         <v>43</v>
       </c>
       <c r="N111" t="str">
-        <f>IF(AND(OR(T111="A", T111="N"), J111="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O111" t="s">
@@ -17181,7 +17171,7 @@
         <v>43</v>
       </c>
       <c r="N112" t="str">
-        <f>IF(AND(OR(T112="A", T112="N"), J112="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O112" t="s">
@@ -17232,7 +17222,7 @@
         <v>43</v>
       </c>
       <c r="N113" t="str">
-        <f>IF(AND(OR(T113="A", T113="N"), J113="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O113" t="s">
@@ -17286,7 +17276,7 @@
         <v>43</v>
       </c>
       <c r="N114" t="str">
-        <f>IF(AND(OR(T114="A", T114="N"), J114="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O114" t="s">
@@ -17346,7 +17336,7 @@
         <v>43</v>
       </c>
       <c r="N115" t="str">
-        <f>IF(AND(OR(T115="A", T115="N"), J115="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O115" t="s">
@@ -17397,7 +17387,7 @@
         <v>43</v>
       </c>
       <c r="N116" t="str">
-        <f>IF(AND(OR(T116="A", T116="N"), J116="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O116" t="s">
@@ -17448,7 +17438,7 @@
         <v>43</v>
       </c>
       <c r="N117" t="str">
-        <f>IF(AND(OR(T117="A", T117="N"), J117="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O117" t="s">
@@ -17499,7 +17489,7 @@
         <v>43</v>
       </c>
       <c r="N118" t="str">
-        <f>IF(AND(OR(T118="A", T118="N"), J118="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O118" t="s">
@@ -17550,7 +17540,7 @@
         <v>43</v>
       </c>
       <c r="N119" t="str">
-        <f>IF(AND(OR(T119="A", T119="N"), J119="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O119" t="s">
@@ -17601,7 +17591,7 @@
         <v>43</v>
       </c>
       <c r="N120" t="str">
-        <f>IF(AND(OR(T120="A", T120="N"), J120="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O120" t="s">
@@ -17652,7 +17642,7 @@
         <v>43</v>
       </c>
       <c r="N121" t="str">
-        <f>IF(AND(OR(T121="A", T121="N"), J121="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O121" t="s">
@@ -17703,7 +17693,7 @@
         <v>43</v>
       </c>
       <c r="N122" t="str">
-        <f>IF(AND(OR(T122="A", T122="N"), J122="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O122" t="s">
@@ -17763,7 +17753,7 @@
         <v>43</v>
       </c>
       <c r="N123" t="str">
-        <f>IF(AND(OR(T123="A", T123="N"), J123="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="P123" t="s">
@@ -17817,7 +17807,7 @@
         <v>43</v>
       </c>
       <c r="N124" t="str">
-        <f>IF(AND(OR(T124="A", T124="N"), J124="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O124" t="s">
@@ -17868,7 +17858,7 @@
         <v>43</v>
       </c>
       <c r="N125" t="str">
-        <f>IF(AND(OR(T125="A", T125="N"), J125="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O125" t="s">
@@ -17922,7 +17912,7 @@
         <v>43</v>
       </c>
       <c r="N126" t="str">
-        <f>IF(AND(OR(T126="A", T126="N"), J126="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O126" t="s">
@@ -17973,7 +17963,7 @@
         <v>43</v>
       </c>
       <c r="N127" t="str">
-        <f>IF(AND(OR(T127="A", T127="N"), J127="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O127" t="s">
@@ -18024,7 +18014,7 @@
         <v>43</v>
       </c>
       <c r="N128" t="str">
-        <f>IF(AND(OR(T128="A", T128="N"), J128="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O128" t="s">
@@ -18075,7 +18065,7 @@
         <v>43</v>
       </c>
       <c r="N129" t="str">
-        <f>IF(AND(OR(T129="A", T129="N"), J129="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="1"/>
         <v>Not Systemic</v>
       </c>
       <c r="O129" t="s">
@@ -18129,7 +18119,7 @@
         <v>43</v>
       </c>
       <c r="N130" t="str">
-        <f>IF(AND(OR(T130="A", T130="N"), J130="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N130:N193" si="2">IF(AND(OR(T130="A", T130="N"), J130="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O130" t="s">
@@ -18180,7 +18170,7 @@
         <v>43</v>
       </c>
       <c r="N131" t="str">
-        <f>IF(AND(OR(T131="A", T131="N"), J131="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O131" t="s">
@@ -18240,7 +18230,7 @@
         <v>43</v>
       </c>
       <c r="N132" t="str">
-        <f>IF(AND(OR(T132="A", T132="N"), J132="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O132" t="s">
@@ -18291,7 +18281,7 @@
         <v>43</v>
       </c>
       <c r="N133" t="str">
-        <f>IF(AND(OR(T133="A", T133="N"), J133="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O133" t="s">
@@ -18342,7 +18332,7 @@
         <v>43</v>
       </c>
       <c r="N134" t="str">
-        <f>IF(AND(OR(T134="A", T134="N"), J134="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O134" t="s">
@@ -18393,7 +18383,7 @@
         <v>43</v>
       </c>
       <c r="N135" t="str">
-        <f>IF(AND(OR(T135="A", T135="N"), J135="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O135" t="s">
@@ -18453,7 +18443,7 @@
         <v>43</v>
       </c>
       <c r="N136" t="str">
-        <f>IF(AND(OR(T136="A", T136="N"), J136="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O136" t="s">
@@ -18513,7 +18503,7 @@
         <v>43</v>
       </c>
       <c r="N137" t="str">
-        <f>IF(AND(OR(T137="A", T137="N"), J137="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O137" t="s">
@@ -18564,7 +18554,7 @@
         <v>43</v>
       </c>
       <c r="N138" t="str">
-        <f>IF(AND(OR(T138="A", T138="N"), J138="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O138" t="s">
@@ -18615,7 +18605,7 @@
         <v>43</v>
       </c>
       <c r="N139" t="str">
-        <f>IF(AND(OR(T139="A", T139="N"), J139="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O139" t="s">
@@ -18675,7 +18665,7 @@
         <v>43</v>
       </c>
       <c r="N140" t="str">
-        <f>IF(AND(OR(T140="A", T140="N"), J140="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O140" t="s">
@@ -18729,7 +18719,7 @@
         <v>43</v>
       </c>
       <c r="N141" t="str">
-        <f>IF(AND(OR(T141="A", T141="N"), J141="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O141" t="s">
@@ -18783,7 +18773,7 @@
         <v>43</v>
       </c>
       <c r="N142" t="str">
-        <f>IF(AND(OR(T142="A", T142="N"), J142="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="P142" t="s">
@@ -18831,7 +18821,7 @@
         <v>43</v>
       </c>
       <c r="N143" t="str">
-        <f>IF(AND(OR(T143="A", T143="N"), J143="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O143" t="s">
@@ -18882,7 +18872,7 @@
         <v>43</v>
       </c>
       <c r="N144" t="str">
-        <f>IF(AND(OR(T144="A", T144="N"), J144="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="T144" t="s">
@@ -18918,7 +18908,7 @@
         <v>43</v>
       </c>
       <c r="N145" t="str">
-        <f>IF(AND(OR(T145="A", T145="N"), J145="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="T145" t="s">
@@ -18954,7 +18944,7 @@
         <v>43</v>
       </c>
       <c r="N146" t="str">
-        <f>IF(AND(OR(T146="A", T146="N"), J146="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="T146" t="s">
@@ -18993,7 +18983,7 @@
         <v>43</v>
       </c>
       <c r="N147" t="str">
-        <f>IF(AND(OR(T147="A", T147="N"), J147="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O147" t="s">
@@ -19035,7 +19025,7 @@
         <v>43</v>
       </c>
       <c r="N148" t="str">
-        <f>IF(AND(OR(T148="A", T148="N"), J148="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O148" t="s">
@@ -19086,7 +19076,7 @@
         <v>43</v>
       </c>
       <c r="N149" t="str">
-        <f>IF(AND(OR(T149="A", T149="N"), J149="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O149" t="s">
@@ -19164,7 +19154,7 @@
         <v>43</v>
       </c>
       <c r="N150" t="str">
-        <f>IF(AND(OR(T150="A", T150="N"), J150="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O150" t="s">
@@ -19242,7 +19232,7 @@
         <v>43</v>
       </c>
       <c r="N151" t="str">
-        <f>IF(AND(OR(T151="A", T151="N"), J151="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O151" t="s">
@@ -19320,7 +19310,7 @@
         <v>43</v>
       </c>
       <c r="N152" t="str">
-        <f>IF(AND(OR(T152="A", T152="N"), J152="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O152" t="s">
@@ -19398,7 +19388,7 @@
         <v>44</v>
       </c>
       <c r="N153" t="str">
-        <f>IF(AND(OR(T153="A", T153="N"), J153="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O153" t="s">
@@ -19476,7 +19466,7 @@
         <v>43</v>
       </c>
       <c r="N154" t="str">
-        <f>IF(AND(OR(T154="A", T154="N"), J154="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O154" t="s">
@@ -19554,7 +19544,7 @@
         <v>43</v>
       </c>
       <c r="N155" t="str">
-        <f>IF(AND(OR(T155="A", T155="N"), J155="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O155" t="s">
@@ -19635,7 +19625,7 @@
         <v>43</v>
       </c>
       <c r="N156" t="str">
-        <f>IF(AND(OR(T156="A", T156="N"), J156="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O156" t="s">
@@ -19716,7 +19706,7 @@
         <v>44</v>
       </c>
       <c r="N157" t="str">
-        <f>IF(AND(OR(T157="A", T157="N"), J157="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O157" t="s">
@@ -19797,7 +19787,7 @@
         <v>44</v>
       </c>
       <c r="N158" t="str">
-        <f>IF(AND(OR(T158="A", T158="N"), J158="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O158" t="s">
@@ -19878,7 +19868,7 @@
         <v>43</v>
       </c>
       <c r="N159" t="str">
-        <f>IF(AND(OR(T159="A", T159="N"), J159="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O159" t="s">
@@ -19959,7 +19949,7 @@
         <v>44</v>
       </c>
       <c r="N160" t="str">
-        <f>IF(AND(OR(T160="A", T160="N"), J160="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O160" t="s">
@@ -20040,7 +20030,7 @@
         <v>44</v>
       </c>
       <c r="N161" t="str">
-        <f>IF(AND(OR(T161="A", T161="N"), J161="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O161" t="s">
@@ -20118,7 +20108,7 @@
         <v>43</v>
       </c>
       <c r="N162" t="str">
-        <f>IF(AND(OR(T162="A", T162="N"), J162="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O162" t="s">
@@ -20196,7 +20186,7 @@
         <v>43</v>
       </c>
       <c r="N163" t="str">
-        <f>IF(AND(OR(T163="A", T163="N"), J163="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O163" t="s">
@@ -20274,7 +20264,7 @@
         <v>43</v>
       </c>
       <c r="N164" t="str">
-        <f>IF(AND(OR(T164="A", T164="N"), J164="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O164" t="s">
@@ -20352,7 +20342,7 @@
         <v>43</v>
       </c>
       <c r="N165" t="str">
-        <f>IF(AND(OR(T165="A", T165="N"), J165="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O165" t="s">
@@ -20430,7 +20420,7 @@
         <v>44</v>
       </c>
       <c r="N166" t="str">
-        <f>IF(AND(OR(T166="A", T166="N"), J166="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O166" t="s">
@@ -20508,7 +20498,7 @@
         <v>44</v>
       </c>
       <c r="N167" t="str">
-        <f>IF(AND(OR(T167="A", T167="N"), J167="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O167" t="s">
@@ -20586,7 +20576,7 @@
         <v>44</v>
       </c>
       <c r="N168" t="str">
-        <f>IF(AND(OR(T168="A", T168="N"), J168="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O168" t="s">
@@ -20664,7 +20654,7 @@
         <v>43</v>
       </c>
       <c r="N169" t="str">
-        <f>IF(AND(OR(T169="A", T169="N"), J169="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O169" t="s">
@@ -20745,7 +20735,7 @@
         <v>43</v>
       </c>
       <c r="N170" t="str">
-        <f>IF(AND(OR(T170="A", T170="N"), J170="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O170" t="s">
@@ -20823,7 +20813,7 @@
         <v>43</v>
       </c>
       <c r="N171" t="str">
-        <f>IF(AND(OR(T171="A", T171="N"), J171="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O171" t="s">
@@ -20901,7 +20891,7 @@
         <v>44</v>
       </c>
       <c r="N172" t="str">
-        <f>IF(AND(OR(T172="A", T172="N"), J172="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O172" t="s">
@@ -20979,7 +20969,7 @@
         <v>44</v>
       </c>
       <c r="N173" t="str">
-        <f>IF(AND(OR(T173="A", T173="N"), J173="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O173" t="s">
@@ -21057,7 +21047,7 @@
         <v>44</v>
       </c>
       <c r="N174" t="str">
-        <f>IF(AND(OR(T174="A", T174="N"), J174="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O174" t="s">
@@ -21135,7 +21125,7 @@
         <v>44</v>
       </c>
       <c r="N175" t="str">
-        <f>IF(AND(OR(T175="A", T175="N"), J175="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O175" t="s">
@@ -21213,7 +21203,7 @@
         <v>44</v>
       </c>
       <c r="N176" t="str">
-        <f>IF(AND(OR(T176="A", T176="N"), J176="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O176" t="s">
@@ -21291,7 +21281,7 @@
         <v>43</v>
       </c>
       <c r="N177" t="str">
-        <f>IF(AND(OR(T177="A", T177="N"), J177="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O177" t="s">
@@ -21369,7 +21359,7 @@
         <v>43</v>
       </c>
       <c r="N178" t="str">
-        <f>IF(AND(OR(T178="A", T178="N"), J178="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O178" t="s">
@@ -21447,7 +21437,7 @@
         <v>44</v>
       </c>
       <c r="N179" t="str">
-        <f>IF(AND(OR(T179="A", T179="N"), J179="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O179" t="s">
@@ -21525,7 +21515,7 @@
         <v>44</v>
       </c>
       <c r="N180" t="str">
-        <f>IF(AND(OR(T180="A", T180="N"), J180="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O180" t="s">
@@ -21606,7 +21596,7 @@
         <v>43</v>
       </c>
       <c r="N181" t="str">
-        <f>IF(AND(OR(T181="A", T181="N"), J181="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O181" t="s">
@@ -21687,7 +21677,7 @@
         <v>43</v>
       </c>
       <c r="N182" t="str">
-        <f>IF(AND(OR(T182="A", T182="N"), J182="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O182" t="s">
@@ -21768,7 +21758,7 @@
         <v>44</v>
       </c>
       <c r="N183" t="str">
-        <f>IF(AND(OR(T183="A", T183="N"), J183="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O183" t="s">
@@ -21849,7 +21839,7 @@
         <v>43</v>
       </c>
       <c r="N184" t="str">
-        <f>IF(AND(OR(T184="A", T184="N"), J184="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O184" t="s">
@@ -21930,7 +21920,7 @@
         <v>43</v>
       </c>
       <c r="N185" t="str">
-        <f>IF(AND(OR(T185="A", T185="N"), J185="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O185" t="s">
@@ -22008,7 +21998,7 @@
         <v>44</v>
       </c>
       <c r="N186" t="str">
-        <f>IF(AND(OR(T186="A", T186="N"), J186="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O186" t="s">
@@ -22086,7 +22076,7 @@
         <v>43</v>
       </c>
       <c r="N187" t="str">
-        <f>IF(AND(OR(T187="A", T187="N"), J187="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O187" t="s">
@@ -22167,7 +22157,7 @@
         <v>43</v>
       </c>
       <c r="N188" t="str">
-        <f>IF(AND(OR(T188="A", T188="N"), J188="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O188" t="s">
@@ -22248,7 +22238,7 @@
         <v>43</v>
       </c>
       <c r="N189" t="str">
-        <f>IF(AND(OR(T189="A", T189="N"), J189="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O189" t="s">
@@ -22329,7 +22319,7 @@
         <v>44</v>
       </c>
       <c r="N190" t="str">
-        <f>IF(AND(OR(T190="A", T190="N"), J190="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O190" t="s">
@@ -22410,7 +22400,7 @@
         <v>44</v>
       </c>
       <c r="N191" t="str">
-        <f>IF(AND(OR(T191="A", T191="N"), J191="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O191" t="s">
@@ -22491,7 +22481,7 @@
         <v>44</v>
       </c>
       <c r="N192" t="str">
-        <f>IF(AND(OR(T192="A", T192="N"), J192="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O192" t="s">
@@ -22572,7 +22562,7 @@
         <v>43</v>
       </c>
       <c r="N193" t="str">
-        <f>IF(AND(OR(T193="A", T193="N"), J193="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="2"/>
         <v>Not Systemic</v>
       </c>
       <c r="O193" t="s">
@@ -22650,7 +22640,7 @@
         <v>43</v>
       </c>
       <c r="N194" t="str">
-        <f>IF(AND(OR(T194="A", T194="N"), J194="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N194:N257" si="3">IF(AND(OR(T194="A", T194="N"), J194="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O194" t="s">
@@ -22728,7 +22718,7 @@
         <v>43</v>
       </c>
       <c r="N195" t="str">
-        <f>IF(AND(OR(T195="A", T195="N"), J195="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O195" t="s">
@@ -22809,7 +22799,7 @@
         <v>43</v>
       </c>
       <c r="N196" t="str">
-        <f>IF(AND(OR(T196="A", T196="N"), J196="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O196" t="s">
@@ -22890,7 +22880,7 @@
         <v>44</v>
       </c>
       <c r="N197" t="str">
-        <f>IF(AND(OR(T197="A", T197="N"), J197="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O197" t="s">
@@ -22971,7 +22961,7 @@
         <v>43</v>
       </c>
       <c r="N198" t="str">
-        <f>IF(AND(OR(T198="A", T198="N"), J198="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O198" t="s">
@@ -23052,7 +23042,7 @@
         <v>44</v>
       </c>
       <c r="N199" t="str">
-        <f>IF(AND(OR(T199="A", T199="N"), J199="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O199" t="s">
@@ -23133,7 +23123,7 @@
         <v>43</v>
       </c>
       <c r="N200" t="str">
-        <f>IF(AND(OR(T200="A", T200="N"), J200="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O200" t="s">
@@ -23214,7 +23204,7 @@
         <v>43</v>
       </c>
       <c r="N201" t="str">
-        <f>IF(AND(OR(T201="A", T201="N"), J201="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O201" t="s">
@@ -23295,7 +23285,7 @@
         <v>43</v>
       </c>
       <c r="N202" t="str">
-        <f>IF(AND(OR(T202="A", T202="N"), J202="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O202" t="s">
@@ -23376,7 +23366,7 @@
         <v>43</v>
       </c>
       <c r="N203" t="str">
-        <f>IF(AND(OR(T203="A", T203="N"), J203="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O203" t="s">
@@ -23457,7 +23447,7 @@
         <v>43</v>
       </c>
       <c r="N204" t="str">
-        <f>IF(AND(OR(T204="A", T204="N"), J204="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O204" t="s">
@@ -23538,7 +23528,7 @@
         <v>43</v>
       </c>
       <c r="N205" t="str">
-        <f>IF(AND(OR(T205="A", T205="N"), J205="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O205" t="s">
@@ -23619,7 +23609,7 @@
         <v>43</v>
       </c>
       <c r="N206" t="str">
-        <f>IF(AND(OR(T206="A", T206="N"), J206="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O206" t="s">
@@ -23700,7 +23690,7 @@
         <v>44</v>
       </c>
       <c r="N207" t="str">
-        <f>IF(AND(OR(T207="A", T207="N"), J207="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O207" t="s">
@@ -23781,7 +23771,7 @@
         <v>44</v>
       </c>
       <c r="N208" t="str">
-        <f>IF(AND(OR(T208="A", T208="N"), J208="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O208" t="s">
@@ -23862,7 +23852,7 @@
         <v>44</v>
       </c>
       <c r="N209" t="str">
-        <f>IF(AND(OR(T209="A", T209="N"), J209="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O209" t="s">
@@ -23943,7 +23933,7 @@
         <v>43</v>
       </c>
       <c r="N210" t="str">
-        <f>IF(AND(OR(T210="A", T210="N"), J210="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O210" t="s">
@@ -24024,7 +24014,7 @@
         <v>43</v>
       </c>
       <c r="N211" t="str">
-        <f>IF(AND(OR(T211="A", T211="N"), J211="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O211" t="s">
@@ -24105,7 +24095,7 @@
         <v>43</v>
       </c>
       <c r="N212" t="str">
-        <f>IF(AND(OR(T212="A", T212="N"), J212="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O212" t="s">
@@ -24186,7 +24176,7 @@
         <v>43</v>
       </c>
       <c r="N213" t="str">
-        <f>IF(AND(OR(T213="A", T213="N"), J213="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O213" t="s">
@@ -24264,7 +24254,7 @@
         <v>43</v>
       </c>
       <c r="N214" t="str">
-        <f>IF(AND(OR(T214="A", T214="N"), J214="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O214" t="s">
@@ -24342,7 +24332,7 @@
         <v>43</v>
       </c>
       <c r="N215" t="str">
-        <f>IF(AND(OR(T215="A", T215="N"), J215="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O215" t="s">
@@ -24423,7 +24413,7 @@
         <v>43</v>
       </c>
       <c r="N216" t="str">
-        <f>IF(AND(OR(T216="A", T216="N"), J216="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O216" t="s">
@@ -24504,7 +24494,7 @@
         <v>44</v>
       </c>
       <c r="N217" t="str">
-        <f>IF(AND(OR(T217="A", T217="N"), J217="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O217" t="s">
@@ -24585,7 +24575,7 @@
         <v>44</v>
       </c>
       <c r="N218" t="str">
-        <f>IF(AND(OR(T218="A", T218="N"), J218="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O218" t="s">
@@ -24666,7 +24656,7 @@
         <v>44</v>
       </c>
       <c r="N219" t="str">
-        <f>IF(AND(OR(T219="A", T219="N"), J219="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O219" t="s">
@@ -24744,7 +24734,7 @@
         <v>43</v>
       </c>
       <c r="N220" t="str">
-        <f>IF(AND(OR(T220="A", T220="N"), J220="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O220" t="s">
@@ -24825,7 +24815,7 @@
         <v>44</v>
       </c>
       <c r="N221" t="str">
-        <f>IF(AND(OR(T221="A", T221="N"), J221="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O221" t="s">
@@ -24906,7 +24896,7 @@
         <v>43</v>
       </c>
       <c r="N222" t="str">
-        <f>IF(AND(OR(T222="A", T222="N"), J222="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O222" t="s">
@@ -24987,7 +24977,7 @@
         <v>43</v>
       </c>
       <c r="N223" t="str">
-        <f>IF(AND(OR(T223="A", T223="N"), J223="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O223" t="s">
@@ -25068,7 +25058,7 @@
         <v>44</v>
       </c>
       <c r="N224" t="str">
-        <f>IF(AND(OR(T224="A", T224="N"), J224="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O224" t="s">
@@ -25149,7 +25139,7 @@
         <v>43</v>
       </c>
       <c r="N225" t="str">
-        <f>IF(AND(OR(T225="A", T225="N"), J225="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O225" t="s">
@@ -25230,7 +25220,7 @@
         <v>43</v>
       </c>
       <c r="N226" t="str">
-        <f>IF(AND(OR(T226="A", T226="N"), J226="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O226" t="s">
@@ -25311,7 +25301,7 @@
         <v>43</v>
       </c>
       <c r="N227" t="str">
-        <f>IF(AND(OR(T227="A", T227="N"), J227="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O227" t="s">
@@ -25392,7 +25382,7 @@
         <v>43</v>
       </c>
       <c r="N228" t="str">
-        <f>IF(AND(OR(T228="A", T228="N"), J228="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O228" t="s">
@@ -25473,7 +25463,7 @@
         <v>43</v>
       </c>
       <c r="N229" t="str">
-        <f>IF(AND(OR(T229="A", T229="N"), J229="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O229" t="s">
@@ -25554,7 +25544,7 @@
         <v>44</v>
       </c>
       <c r="N230" t="str">
-        <f>IF(AND(OR(T230="A", T230="N"), J230="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O230" t="s">
@@ -25635,7 +25625,7 @@
         <v>44</v>
       </c>
       <c r="N231" t="str">
-        <f>IF(AND(OR(T231="A", T231="N"), J231="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O231" t="s">
@@ -25716,7 +25706,7 @@
         <v>44</v>
       </c>
       <c r="N232" t="str">
-        <f>IF(AND(OR(T232="A", T232="N"), J232="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O232" t="s">
@@ -25797,7 +25787,7 @@
         <v>43</v>
       </c>
       <c r="N233" t="str">
-        <f>IF(AND(OR(T233="A", T233="N"), J233="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O233" t="s">
@@ -25878,7 +25868,7 @@
         <v>43</v>
       </c>
       <c r="N234" t="str">
-        <f>IF(AND(OR(T234="A", T234="N"), J234="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O234" t="s">
@@ -25959,7 +25949,7 @@
         <v>44</v>
       </c>
       <c r="N235" t="str">
-        <f>IF(AND(OR(T235="A", T235="N"), J235="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O235" t="s">
@@ -26040,7 +26030,7 @@
         <v>44</v>
       </c>
       <c r="N236" t="str">
-        <f>IF(AND(OR(T236="A", T236="N"), J236="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O236" t="s">
@@ -26121,7 +26111,7 @@
         <v>43</v>
       </c>
       <c r="N237" t="str">
-        <f>IF(AND(OR(T237="A", T237="N"), J237="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O237" t="s">
@@ -26202,7 +26192,7 @@
         <v>44</v>
       </c>
       <c r="N238" t="str">
-        <f>IF(AND(OR(T238="A", T238="N"), J238="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O238" t="s">
@@ -26283,7 +26273,7 @@
         <v>43</v>
       </c>
       <c r="N239" t="str">
-        <f>IF(AND(OR(T239="A", T239="N"), J239="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O239" t="s">
@@ -26364,7 +26354,7 @@
         <v>43</v>
       </c>
       <c r="N240" t="str">
-        <f>IF(AND(OR(T240="A", T240="N"), J240="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O240" t="s">
@@ -26442,7 +26432,7 @@
         <v>44</v>
       </c>
       <c r="N241" t="str">
-        <f>IF(AND(OR(T241="A", T241="N"), J241="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O241" t="s">
@@ -26520,7 +26510,7 @@
         <v>43</v>
       </c>
       <c r="N242" t="str">
-        <f>IF(AND(OR(T242="A", T242="N"), J242="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O242" t="s">
@@ -26598,7 +26588,7 @@
         <v>43</v>
       </c>
       <c r="N243" t="str">
-        <f>IF(AND(OR(T243="A", T243="N"), J243="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O243" t="s">
@@ -26676,7 +26666,7 @@
         <v>44</v>
       </c>
       <c r="N244" t="str">
-        <f>IF(AND(OR(T244="A", T244="N"), J244="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O244" t="s">
@@ -26754,7 +26744,7 @@
         <v>43</v>
       </c>
       <c r="N245" t="str">
-        <f>IF(AND(OR(T245="A", T245="N"), J245="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O245" t="s">
@@ -26835,7 +26825,7 @@
         <v>44</v>
       </c>
       <c r="N246" t="str">
-        <f>IF(AND(OR(T246="A", T246="N"), J246="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O246" t="s">
@@ -26916,7 +26906,7 @@
         <v>44</v>
       </c>
       <c r="N247" t="str">
-        <f>IF(AND(OR(T247="A", T247="N"), J247="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O247" t="s">
@@ -26994,7 +26984,7 @@
         <v>44</v>
       </c>
       <c r="N248" t="str">
-        <f>IF(AND(OR(T248="A", T248="N"), J248="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O248" t="s">
@@ -27078,7 +27068,7 @@
         <v>44</v>
       </c>
       <c r="N249" t="str">
-        <f>IF(AND(OR(T249="A", T249="N"), J249="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O249" t="s">
@@ -27159,7 +27149,7 @@
         <v>43</v>
       </c>
       <c r="N250" t="str">
-        <f>IF(AND(OR(T250="A", T250="N"), J250="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O250" t="s">
@@ -27237,7 +27227,7 @@
         <v>44</v>
       </c>
       <c r="N251" t="str">
-        <f>IF(AND(OR(T251="A", T251="N"), J251="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O251" t="s">
@@ -27315,7 +27305,7 @@
         <v>44</v>
       </c>
       <c r="N252" t="str">
-        <f>IF(AND(OR(T252="A", T252="N"), J252="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O252" t="s">
@@ -27396,7 +27386,7 @@
         <v>44</v>
       </c>
       <c r="N253" t="str">
-        <f>IF(AND(OR(T253="A", T253="N"), J253="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O253" t="s">
@@ -27477,7 +27467,7 @@
         <v>44</v>
       </c>
       <c r="N254" t="str">
-        <f>IF(AND(OR(T254="A", T254="N"), J254="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O254" t="s">
@@ -27558,7 +27548,7 @@
         <v>44</v>
       </c>
       <c r="N255" t="str">
-        <f>IF(AND(OR(T255="A", T255="N"), J255="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O255" t="s">
@@ -27639,7 +27629,7 @@
         <v>43</v>
       </c>
       <c r="N256" t="str">
-        <f>IF(AND(OR(T256="A", T256="N"), J256="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O256" t="s">
@@ -27720,7 +27710,7 @@
         <v>44</v>
       </c>
       <c r="N257" t="str">
-        <f>IF(AND(OR(T257="A", T257="N"), J257="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="3"/>
         <v>Not Systemic</v>
       </c>
       <c r="O257" t="s">
@@ -27801,7 +27791,7 @@
         <v>43</v>
       </c>
       <c r="N258" t="str">
-        <f>IF(AND(OR(T258="A", T258="N"), J258="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N258:N321" si="4">IF(AND(OR(T258="A", T258="N"), J258="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O258" t="s">
@@ -27882,7 +27872,7 @@
         <v>43</v>
       </c>
       <c r="N259" t="str">
-        <f>IF(AND(OR(T259="A", T259="N"), J259="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O259" t="s">
@@ -27963,7 +27953,7 @@
         <v>44</v>
       </c>
       <c r="N260" t="str">
-        <f>IF(AND(OR(T260="A", T260="N"), J260="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O260" t="s">
@@ -28044,7 +28034,7 @@
         <v>43</v>
       </c>
       <c r="N261" t="str">
-        <f>IF(AND(OR(T261="A", T261="N"), J261="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O261" t="s">
@@ -28125,7 +28115,7 @@
         <v>43</v>
       </c>
       <c r="N262" t="str">
-        <f>IF(AND(OR(T262="A", T262="N"), J262="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O262" t="s">
@@ -28206,7 +28196,7 @@
         <v>44</v>
       </c>
       <c r="N263" t="str">
-        <f>IF(AND(OR(T263="A", T263="N"), J263="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O263" t="s">
@@ -28287,7 +28277,7 @@
         <v>43</v>
       </c>
       <c r="N264" t="str">
-        <f>IF(AND(OR(T264="A", T264="N"), J264="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O264" t="s">
@@ -28365,7 +28355,7 @@
         <v>43</v>
       </c>
       <c r="N265" t="str">
-        <f>IF(AND(OR(T265="A", T265="N"), J265="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O265" t="s">
@@ -28446,7 +28436,7 @@
         <v>43</v>
       </c>
       <c r="N266" t="str">
-        <f>IF(AND(OR(T266="A", T266="N"), J266="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O266" t="s">
@@ -28527,7 +28517,7 @@
         <v>43</v>
       </c>
       <c r="N267" t="str">
-        <f>IF(AND(OR(T267="A", T267="N"), J267="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O267" t="s">
@@ -28605,7 +28595,7 @@
         <v>43</v>
       </c>
       <c r="N268" t="str">
-        <f>IF(AND(OR(T268="A", T268="N"), J268="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O268" t="s">
@@ -28686,7 +28676,7 @@
         <v>43</v>
       </c>
       <c r="N269" t="str">
-        <f>IF(AND(OR(T269="A", T269="N"), J269="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O269" t="s">
@@ -28767,7 +28757,7 @@
         <v>44</v>
       </c>
       <c r="N270" t="str">
-        <f>IF(AND(OR(T270="A", T270="N"), J270="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O270" t="s">
@@ -28848,7 +28838,7 @@
         <v>43</v>
       </c>
       <c r="N271" t="str">
-        <f>IF(AND(OR(T271="A", T271="N"), J271="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O271" t="s">
@@ -28929,7 +28919,7 @@
         <v>43</v>
       </c>
       <c r="N272" t="str">
-        <f>IF(AND(OR(T272="A", T272="N"), J272="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O272" t="s">
@@ -29010,7 +29000,7 @@
         <v>43</v>
       </c>
       <c r="N273" t="str">
-        <f>IF(AND(OR(T273="A", T273="N"), J273="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O273" t="s">
@@ -29088,7 +29078,7 @@
         <v>44</v>
       </c>
       <c r="N274" t="str">
-        <f>IF(AND(OR(T274="A", T274="N"), J274="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O274" t="s">
@@ -29169,7 +29159,7 @@
         <v>43</v>
       </c>
       <c r="N275" t="str">
-        <f>IF(AND(OR(T275="A", T275="N"), J275="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O275" t="s">
@@ -29250,7 +29240,7 @@
         <v>43</v>
       </c>
       <c r="N276" t="str">
-        <f>IF(AND(OR(T276="A", T276="N"), J276="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O276" t="s">
@@ -29331,7 +29321,7 @@
         <v>43</v>
       </c>
       <c r="N277" t="str">
-        <f>IF(AND(OR(T277="A", T277="N"), J277="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O277" t="s">
@@ -29412,7 +29402,7 @@
         <v>44</v>
       </c>
       <c r="N278" t="str">
-        <f>IF(AND(OR(T278="A", T278="N"), J278="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O278" t="s">
@@ -29493,7 +29483,7 @@
         <v>43</v>
       </c>
       <c r="N279" t="str">
-        <f>IF(AND(OR(T279="A", T279="N"), J279="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O279" t="s">
@@ -29574,7 +29564,7 @@
         <v>44</v>
       </c>
       <c r="N280" t="str">
-        <f>IF(AND(OR(T280="A", T280="N"), J280="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O280" t="s">
@@ -29655,7 +29645,7 @@
         <v>44</v>
       </c>
       <c r="N281" t="str">
-        <f>IF(AND(OR(T281="A", T281="N"), J281="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O281" t="s">
@@ -29736,7 +29726,7 @@
         <v>44</v>
       </c>
       <c r="N282" t="str">
-        <f>IF(AND(OR(T282="A", T282="N"), J282="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O282" t="s">
@@ -29817,7 +29807,7 @@
         <v>43</v>
       </c>
       <c r="N283" t="str">
-        <f>IF(AND(OR(T283="A", T283="N"), J283="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O283" t="s">
@@ -29898,7 +29888,7 @@
         <v>43</v>
       </c>
       <c r="N284" t="str">
-        <f>IF(AND(OR(T284="A", T284="N"), J284="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O284" t="s">
@@ -29982,7 +29972,7 @@
         <v>44</v>
       </c>
       <c r="N285" t="str">
-        <f>IF(AND(OR(T285="A", T285="N"), J285="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O285" t="s">
@@ -30063,7 +30053,7 @@
         <v>44</v>
       </c>
       <c r="N286" t="str">
-        <f>IF(AND(OR(T286="A", T286="N"), J286="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O286" t="s">
@@ -30144,7 +30134,7 @@
         <v>43</v>
       </c>
       <c r="N287" t="str">
-        <f>IF(AND(OR(T287="A", T287="N"), J287="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O287" t="s">
@@ -30225,7 +30215,7 @@
         <v>43</v>
       </c>
       <c r="N288" t="str">
-        <f>IF(AND(OR(T288="A", T288="N"), J288="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O288" t="s">
@@ -30306,7 +30296,7 @@
         <v>43</v>
       </c>
       <c r="N289" t="str">
-        <f>IF(AND(OR(T289="A", T289="N"), J289="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O289" t="s">
@@ -30387,7 +30377,7 @@
         <v>44</v>
       </c>
       <c r="N290" t="str">
-        <f>IF(AND(OR(T290="A", T290="N"), J290="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O290" t="s">
@@ -30468,7 +30458,7 @@
         <v>44</v>
       </c>
       <c r="N291" t="str">
-        <f>IF(AND(OR(T291="A", T291="N"), J291="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O291" t="s">
@@ -30549,7 +30539,7 @@
         <v>44</v>
       </c>
       <c r="N292" t="str">
-        <f>IF(AND(OR(T292="A", T292="N"), J292="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O292" t="s">
@@ -30630,7 +30620,7 @@
         <v>43</v>
       </c>
       <c r="N293" t="str">
-        <f>IF(AND(OR(T293="A", T293="N"), J293="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O293" t="s">
@@ -30711,7 +30701,7 @@
         <v>43</v>
       </c>
       <c r="N294" t="str">
-        <f>IF(AND(OR(T294="A", T294="N"), J294="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O294" t="s">
@@ -30792,7 +30782,7 @@
         <v>43</v>
       </c>
       <c r="N295" t="str">
-        <f>IF(AND(OR(T295="A", T295="N"), J295="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O295" t="s">
@@ -30870,7 +30860,7 @@
         <v>43</v>
       </c>
       <c r="N296" t="str">
-        <f>IF(AND(OR(T296="A", T296="N"), J296="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O296" t="s">
@@ -30948,7 +30938,7 @@
         <v>44</v>
       </c>
       <c r="N297" t="str">
-        <f>IF(AND(OR(T297="A", T297="N"), J297="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O297" t="s">
@@ -31029,7 +31019,7 @@
         <v>43</v>
       </c>
       <c r="N298" t="str">
-        <f>IF(AND(OR(T298="A", T298="N"), J298="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O298" t="s">
@@ -31110,7 +31100,7 @@
         <v>44</v>
       </c>
       <c r="N299" t="str">
-        <f>IF(AND(OR(T299="A", T299="N"), J299="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O299" t="s">
@@ -31191,7 +31181,7 @@
         <v>43</v>
       </c>
       <c r="N300" t="str">
-        <f>IF(AND(OR(T300="A", T300="N"), J300="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O300" t="s">
@@ -31272,7 +31262,7 @@
         <v>43</v>
       </c>
       <c r="N301" t="str">
-        <f>IF(AND(OR(T301="A", T301="N"), J301="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O301" t="s">
@@ -31353,7 +31343,7 @@
         <v>44</v>
       </c>
       <c r="N302" t="str">
-        <f>IF(AND(OR(T302="A", T302="N"), J302="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O302" t="s">
@@ -31434,7 +31424,7 @@
         <v>44</v>
       </c>
       <c r="N303" t="str">
-        <f>IF(AND(OR(T303="A", T303="N"), J303="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O303" t="s">
@@ -31515,7 +31505,7 @@
         <v>44</v>
       </c>
       <c r="N304" t="str">
-        <f>IF(AND(OR(T304="A", T304="N"), J304="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O304" t="s">
@@ -31596,7 +31586,7 @@
         <v>44</v>
       </c>
       <c r="N305" t="str">
-        <f>IF(AND(OR(T305="A", T305="N"), J305="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O305" t="s">
@@ -31674,7 +31664,7 @@
         <v>43</v>
       </c>
       <c r="N306" t="str">
-        <f>IF(AND(OR(T306="A", T306="N"), J306="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O306" t="s">
@@ -31752,7 +31742,7 @@
         <v>44</v>
       </c>
       <c r="N307" t="str">
-        <f>IF(AND(OR(T307="A", T307="N"), J307="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O307" t="s">
@@ -31830,7 +31820,7 @@
         <v>43</v>
       </c>
       <c r="N308" t="str">
-        <f>IF(AND(OR(T308="A", T308="N"), J308="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O308" t="s">
@@ -31908,7 +31898,7 @@
         <v>44</v>
       </c>
       <c r="N309" t="str">
-        <f>IF(AND(OR(T309="A", T309="N"), J309="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O309" t="s">
@@ -31986,7 +31976,7 @@
         <v>43</v>
       </c>
       <c r="N310" t="str">
-        <f>IF(AND(OR(T310="A", T310="N"), J310="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O310" t="s">
@@ -32064,7 +32054,7 @@
         <v>43</v>
       </c>
       <c r="N311" t="str">
-        <f>IF(AND(OR(T311="A", T311="N"), J311="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O311" t="s">
@@ -32145,7 +32135,7 @@
         <v>44</v>
       </c>
       <c r="N312" t="str">
-        <f>IF(AND(OR(T312="A", T312="N"), J312="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O312" t="s">
@@ -32226,7 +32216,7 @@
         <v>44</v>
       </c>
       <c r="N313" t="str">
-        <f>IF(AND(OR(T313="A", T313="N"), J313="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O313" t="s">
@@ -32307,7 +32297,7 @@
         <v>43</v>
       </c>
       <c r="N314" t="str">
-        <f>IF(AND(OR(T314="A", T314="N"), J314="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O314" t="s">
@@ -32388,7 +32378,7 @@
         <v>44</v>
       </c>
       <c r="N315" t="str">
-        <f>IF(AND(OR(T315="A", T315="N"), J315="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O315" t="s">
@@ -32469,7 +32459,7 @@
         <v>44</v>
       </c>
       <c r="N316" t="str">
-        <f>IF(AND(OR(T316="A", T316="N"), J316="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O316" t="s">
@@ -32550,7 +32540,7 @@
         <v>44</v>
       </c>
       <c r="N317" t="str">
-        <f>IF(AND(OR(T317="A", T317="N"), J317="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O317" t="s">
@@ -32631,7 +32621,7 @@
         <v>44</v>
       </c>
       <c r="N318" t="str">
-        <f>IF(AND(OR(T318="A", T318="N"), J318="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O318" t="s">
@@ -32712,7 +32702,7 @@
         <v>44</v>
       </c>
       <c r="N319" t="str">
-        <f>IF(AND(OR(T319="A", T319="N"), J319="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O319" t="s">
@@ -32793,7 +32783,7 @@
         <v>43</v>
       </c>
       <c r="N320" t="str">
-        <f>IF(AND(OR(T320="A", T320="N"), J320="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O320" t="s">
@@ -32874,7 +32864,7 @@
         <v>43</v>
       </c>
       <c r="N321" t="str">
-        <f>IF(AND(OR(T321="A", T321="N"), J321="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="4"/>
         <v>Not Systemic</v>
       </c>
       <c r="O321" t="s">
@@ -32952,7 +32942,7 @@
         <v>44</v>
       </c>
       <c r="N322" t="str">
-        <f>IF(AND(OR(T322="A", T322="N"), J322="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N322:N385" si="5">IF(AND(OR(T322="A", T322="N"), J322="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O322" t="s">
@@ -33033,7 +33023,7 @@
         <v>44</v>
       </c>
       <c r="N323" t="str">
-        <f>IF(AND(OR(T323="A", T323="N"), J323="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O323" t="s">
@@ -33117,7 +33107,7 @@
         <v>44</v>
       </c>
       <c r="N324" t="str">
-        <f>IF(AND(OR(T324="A", T324="N"), J324="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O324" t="s">
@@ -33198,7 +33188,7 @@
         <v>44</v>
       </c>
       <c r="N325" t="str">
-        <f>IF(AND(OR(T325="A", T325="N"), J325="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O325" t="s">
@@ -33279,7 +33269,7 @@
         <v>44</v>
       </c>
       <c r="N326" t="str">
-        <f>IF(AND(OR(T326="A", T326="N"), J326="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O326" t="s">
@@ -33363,7 +33353,7 @@
         <v>44</v>
       </c>
       <c r="N327" t="str">
-        <f>IF(AND(OR(T327="A", T327="N"), J327="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O327" t="s">
@@ -33447,7 +33437,7 @@
         <v>44</v>
       </c>
       <c r="N328" t="str">
-        <f>IF(AND(OR(T328="A", T328="N"), J328="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O328" t="s">
@@ -33531,7 +33521,7 @@
         <v>44</v>
       </c>
       <c r="N329" t="str">
-        <f>IF(AND(OR(T329="A", T329="N"), J329="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O329" t="s">
@@ -33612,7 +33602,7 @@
         <v>44</v>
       </c>
       <c r="N330" t="str">
-        <f>IF(AND(OR(T330="A", T330="N"), J330="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O330" t="s">
@@ -33693,7 +33683,7 @@
         <v>44</v>
       </c>
       <c r="N331" t="str">
-        <f>IF(AND(OR(T331="A", T331="N"), J331="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O331" t="s">
@@ -33774,7 +33764,7 @@
         <v>43</v>
       </c>
       <c r="N332" t="str">
-        <f>IF(AND(OR(T332="A", T332="N"), J332="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O332" t="s">
@@ -33855,7 +33845,7 @@
         <v>44</v>
       </c>
       <c r="N333" t="str">
-        <f>IF(AND(OR(T333="A", T333="N"), J333="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O333" t="s">
@@ -33936,7 +33926,7 @@
         <v>43</v>
       </c>
       <c r="N334" t="str">
-        <f>IF(AND(OR(T334="A", T334="N"), J334="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O334" t="s">
@@ -34014,7 +34004,7 @@
         <v>44</v>
       </c>
       <c r="N335" t="str">
-        <f>IF(AND(OR(T335="A", T335="N"), J335="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O335" t="s">
@@ -34092,7 +34082,7 @@
         <v>44</v>
       </c>
       <c r="N336" t="str">
-        <f>IF(AND(OR(T336="A", T336="N"), J336="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O336" t="s">
@@ -34170,7 +34160,7 @@
         <v>43</v>
       </c>
       <c r="N337" t="str">
-        <f>IF(AND(OR(T337="A", T337="N"), J337="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O337" t="s">
@@ -34248,7 +34238,7 @@
         <v>43</v>
       </c>
       <c r="N338" t="str">
-        <f>IF(AND(OR(T338="A", T338="N"), J338="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O338" t="s">
@@ -34326,7 +34316,7 @@
         <v>43</v>
       </c>
       <c r="N339" t="str">
-        <f>IF(AND(OR(T339="A", T339="N"), J339="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O339" t="s">
@@ -34407,7 +34397,7 @@
         <v>43</v>
       </c>
       <c r="N340" t="str">
-        <f>IF(AND(OR(T340="A", T340="N"), J340="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O340" t="s">
@@ -34491,7 +34481,7 @@
         <v>43</v>
       </c>
       <c r="N341" t="str">
-        <f>IF(AND(OR(T341="A", T341="N"), J341="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O341" t="s">
@@ -34578,7 +34568,7 @@
         <v>43</v>
       </c>
       <c r="N342" t="str">
-        <f>IF(AND(OR(T342="A", T342="N"), J342="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O342" t="s">
@@ -34659,7 +34649,7 @@
         <v>44</v>
       </c>
       <c r="N343" t="str">
-        <f>IF(AND(OR(T343="A", T343="N"), J343="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O343" t="s">
@@ -34743,7 +34733,7 @@
         <v>44</v>
       </c>
       <c r="N344" t="str">
-        <f>IF(AND(OR(T344="A", T344="N"), J344="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O344" t="s">
@@ -34827,7 +34817,7 @@
         <v>43</v>
       </c>
       <c r="N345" t="str">
-        <f>IF(AND(OR(T345="A", T345="N"), J345="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O345" t="s">
@@ -34911,7 +34901,7 @@
         <v>43</v>
       </c>
       <c r="N346" t="str">
-        <f>IF(AND(OR(T346="A", T346="N"), J346="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O346" t="s">
@@ -34992,7 +34982,7 @@
         <v>44</v>
       </c>
       <c r="N347" t="str">
-        <f>IF(AND(OR(T347="A", T347="N"), J347="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O347" t="s">
@@ -35073,7 +35063,7 @@
         <v>44</v>
       </c>
       <c r="N348" t="str">
-        <f>IF(AND(OR(T348="A", T348="N"), J348="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O348" t="s">
@@ -35154,7 +35144,7 @@
         <v>44</v>
       </c>
       <c r="N349" t="str">
-        <f>IF(AND(OR(T349="A", T349="N"), J349="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O349" t="s">
@@ -35235,7 +35225,7 @@
         <v>44</v>
       </c>
       <c r="N350" t="str">
-        <f>IF(AND(OR(T350="A", T350="N"), J350="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O350" t="s">
@@ -35313,7 +35303,7 @@
         <v>43</v>
       </c>
       <c r="N351" t="str">
-        <f>IF(AND(OR(T351="A", T351="N"), J351="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O351" t="s">
@@ -35391,7 +35381,7 @@
         <v>44</v>
       </c>
       <c r="N352" t="str">
-        <f>IF(AND(OR(T352="A", T352="N"), J352="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O352" t="s">
@@ -35469,7 +35459,7 @@
         <v>44</v>
       </c>
       <c r="N353" t="str">
-        <f>IF(AND(OR(T353="A", T353="N"), J353="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O353" t="s">
@@ -35547,7 +35537,7 @@
         <v>44</v>
       </c>
       <c r="N354" t="str">
-        <f>IF(AND(OR(T354="A", T354="N"), J354="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O354" t="s">
@@ -35625,7 +35615,7 @@
         <v>43</v>
       </c>
       <c r="N355" t="str">
-        <f>IF(AND(OR(T355="A", T355="N"), J355="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O355" t="s">
@@ -35706,7 +35696,7 @@
         <v>44</v>
       </c>
       <c r="N356" t="str">
-        <f>IF(AND(OR(T356="A", T356="N"), J356="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O356" t="s">
@@ -35787,7 +35777,7 @@
         <v>44</v>
       </c>
       <c r="N357" t="str">
-        <f>IF(AND(OR(T357="A", T357="N"), J357="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O357" t="s">
@@ -35868,7 +35858,7 @@
         <v>43</v>
       </c>
       <c r="N358" t="str">
-        <f>IF(AND(OR(T358="A", T358="N"), J358="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O358" t="s">
@@ -35946,7 +35936,7 @@
         <v>43</v>
       </c>
       <c r="N359" t="str">
-        <f>IF(AND(OR(T359="A", T359="N"), J359="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O359" t="s">
@@ -36027,7 +36017,7 @@
         <v>44</v>
       </c>
       <c r="N360" t="str">
-        <f>IF(AND(OR(T360="A", T360="N"), J360="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O360" t="s">
@@ -36108,7 +36098,7 @@
         <v>43</v>
       </c>
       <c r="N361" t="str">
-        <f>IF(AND(OR(T361="A", T361="N"), J361="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O361" t="s">
@@ -36189,7 +36179,7 @@
         <v>44</v>
       </c>
       <c r="N362" t="str">
-        <f>IF(AND(OR(T362="A", T362="N"), J362="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O362" t="s">
@@ -36270,7 +36260,7 @@
         <v>43</v>
       </c>
       <c r="N363" t="str">
-        <f>IF(AND(OR(T363="A", T363="N"), J363="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O363" t="s">
@@ -36351,7 +36341,7 @@
         <v>44</v>
       </c>
       <c r="N364" t="str">
-        <f>IF(AND(OR(T364="A", T364="N"), J364="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O364" t="s">
@@ -36432,7 +36422,7 @@
         <v>44</v>
       </c>
       <c r="N365" t="str">
-        <f>IF(AND(OR(T365="A", T365="N"), J365="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O365" t="s">
@@ -36513,7 +36503,7 @@
         <v>43</v>
       </c>
       <c r="N366" t="str">
-        <f>IF(AND(OR(T366="A", T366="N"), J366="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O366" t="s">
@@ -36594,7 +36584,7 @@
         <v>44</v>
       </c>
       <c r="N367" t="str">
-        <f>IF(AND(OR(T367="A", T367="N"), J367="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O367" t="s">
@@ -36675,7 +36665,7 @@
         <v>44</v>
       </c>
       <c r="N368" t="str">
-        <f>IF(AND(OR(T368="A", T368="N"), J368="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O368" t="s">
@@ -36759,7 +36749,7 @@
         <v>44</v>
       </c>
       <c r="N369" t="str">
-        <f>IF(AND(OR(T369="A", T369="N"), J369="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O369" t="s">
@@ -36840,7 +36830,7 @@
         <v>44</v>
       </c>
       <c r="N370" t="str">
-        <f>IF(AND(OR(T370="A", T370="N"), J370="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O370" t="s">
@@ -36918,7 +36908,7 @@
         <v>44</v>
       </c>
       <c r="N371" t="str">
-        <f>IF(AND(OR(T371="A", T371="N"), J371="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O371" t="s">
@@ -37002,7 +36992,7 @@
         <v>44</v>
       </c>
       <c r="N372" t="str">
-        <f>IF(AND(OR(T372="A", T372="N"), J372="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O372" t="s">
@@ -37083,7 +37073,7 @@
         <v>44</v>
       </c>
       <c r="N373" t="str">
-        <f>IF(AND(OR(T373="A", T373="N"), J373="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O373" t="s">
@@ -37164,7 +37154,7 @@
         <v>43</v>
       </c>
       <c r="N374" t="str">
-        <f>IF(AND(OR(T374="A", T374="N"), J374="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O374" t="s">
@@ -37245,7 +37235,7 @@
         <v>43</v>
       </c>
       <c r="N375" t="str">
-        <f>IF(AND(OR(T375="A", T375="N"), J375="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O375" t="s">
@@ -37326,7 +37316,7 @@
         <v>44</v>
       </c>
       <c r="N376" t="str">
-        <f>IF(AND(OR(T376="A", T376="N"), J376="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O376" t="s">
@@ -37407,7 +37397,7 @@
         <v>43</v>
       </c>
       <c r="N377" t="str">
-        <f>IF(AND(OR(T377="A", T377="N"), J377="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O377" t="s">
@@ -37491,7 +37481,7 @@
         <v>44</v>
       </c>
       <c r="N378" t="str">
-        <f>IF(AND(OR(T378="A", T378="N"), J378="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O378" t="s">
@@ -37572,7 +37562,7 @@
         <v>44</v>
       </c>
       <c r="N379" t="str">
-        <f>IF(AND(OR(T379="A", T379="N"), J379="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O379" t="s">
@@ -37650,7 +37640,7 @@
         <v>43</v>
       </c>
       <c r="N380" t="str">
-        <f>IF(AND(OR(T380="A", T380="N"), J380="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O380" t="s">
@@ -37731,7 +37721,7 @@
         <v>44</v>
       </c>
       <c r="N381" t="str">
-        <f>IF(AND(OR(T381="A", T381="N"), J381="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O381" t="s">
@@ -37812,7 +37802,7 @@
         <v>44</v>
       </c>
       <c r="N382" t="str">
-        <f>IF(AND(OR(T382="A", T382="N"), J382="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O382" t="s">
@@ -37893,7 +37883,7 @@
         <v>44</v>
       </c>
       <c r="N383" t="str">
-        <f>IF(AND(OR(T383="A", T383="N"), J383="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O383" t="s">
@@ -37974,7 +37964,7 @@
         <v>43</v>
       </c>
       <c r="N384" t="str">
-        <f>IF(AND(OR(T384="A", T384="N"), J384="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O384" t="s">
@@ -38055,7 +38045,7 @@
         <v>44</v>
       </c>
       <c r="N385" t="str">
-        <f>IF(AND(OR(T385="A", T385="N"), J385="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="5"/>
         <v>Not Systemic</v>
       </c>
       <c r="O385" t="s">
@@ -38136,7 +38126,7 @@
         <v>44</v>
       </c>
       <c r="N386" t="str">
-        <f>IF(AND(OR(T386="A", T386="N"), J386="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N386:N449" si="6">IF(AND(OR(T386="A", T386="N"), J386="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O386" t="s">
@@ -38217,7 +38207,7 @@
         <v>44</v>
       </c>
       <c r="N387" t="str">
-        <f>IF(AND(OR(T387="A", T387="N"), J387="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O387" t="s">
@@ -38295,7 +38285,7 @@
         <v>44</v>
       </c>
       <c r="N388" t="str">
-        <f>IF(AND(OR(T388="A", T388="N"), J388="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O388" t="s">
@@ -38376,7 +38366,7 @@
         <v>44</v>
       </c>
       <c r="N389" t="str">
-        <f>IF(AND(OR(T389="A", T389="N"), J389="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O389" t="s">
@@ -38457,7 +38447,7 @@
         <v>44</v>
       </c>
       <c r="N390" t="str">
-        <f>IF(AND(OR(T390="A", T390="N"), J390="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O390" t="s">
@@ -38538,7 +38528,7 @@
         <v>44</v>
       </c>
       <c r="N391" t="str">
-        <f>IF(AND(OR(T391="A", T391="N"), J391="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O391" t="s">
@@ -38622,7 +38612,7 @@
         <v>44</v>
       </c>
       <c r="N392" t="str">
-        <f>IF(AND(OR(T392="A", T392="N"), J392="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O392" t="s">
@@ -38703,7 +38693,7 @@
         <v>44</v>
       </c>
       <c r="N393" t="str">
-        <f>IF(AND(OR(T393="A", T393="N"), J393="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O393" t="s">
@@ -38784,7 +38774,7 @@
         <v>44</v>
       </c>
       <c r="N394" t="str">
-        <f>IF(AND(OR(T394="A", T394="N"), J394="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O394" t="s">
@@ -38865,7 +38855,7 @@
         <v>43</v>
       </c>
       <c r="N395" t="str">
-        <f>IF(AND(OR(T395="A", T395="N"), J395="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O395" t="s">
@@ -38946,7 +38936,7 @@
         <v>43</v>
       </c>
       <c r="N396" t="str">
-        <f>IF(AND(OR(T396="A", T396="N"), J396="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O396" t="s">
@@ -39027,7 +39017,7 @@
         <v>43</v>
       </c>
       <c r="N397" t="str">
-        <f>IF(AND(OR(T397="A", T397="N"), J397="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O397" t="s">
@@ -39108,7 +39098,7 @@
         <v>44</v>
       </c>
       <c r="N398" t="str">
-        <f>IF(AND(OR(T398="A", T398="N"), J398="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O398" t="s">
@@ -39189,7 +39179,7 @@
         <v>44</v>
       </c>
       <c r="N399" t="str">
-        <f>IF(AND(OR(T399="A", T399="N"), J399="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O399" t="s">
@@ -39270,7 +39260,7 @@
         <v>44</v>
       </c>
       <c r="N400" t="str">
-        <f>IF(AND(OR(T400="A", T400="N"), J400="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O400" t="s">
@@ -39351,7 +39341,7 @@
         <v>44</v>
       </c>
       <c r="N401" t="str">
-        <f>IF(AND(OR(T401="A", T401="N"), J401="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O401" t="s">
@@ -39432,7 +39422,7 @@
         <v>43</v>
       </c>
       <c r="N402" t="str">
-        <f>IF(AND(OR(T402="A", T402="N"), J402="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O402" t="s">
@@ -39513,7 +39503,7 @@
         <v>44</v>
       </c>
       <c r="N403" t="str">
-        <f>IF(AND(OR(T403="A", T403="N"), J403="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O403" t="s">
@@ -39594,7 +39584,7 @@
         <v>44</v>
       </c>
       <c r="N404" t="str">
-        <f>IF(AND(OR(T404="A", T404="N"), J404="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O404" t="s">
@@ -39675,7 +39665,7 @@
         <v>44</v>
       </c>
       <c r="N405" t="str">
-        <f>IF(AND(OR(T405="A", T405="N"), J405="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O405" t="s">
@@ -39753,7 +39743,7 @@
         <v>44</v>
       </c>
       <c r="N406" t="str">
-        <f>IF(AND(OR(T406="A", T406="N"), J406="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O406" t="s">
@@ -39834,7 +39824,7 @@
         <v>44</v>
       </c>
       <c r="N407" t="str">
-        <f>IF(AND(OR(T407="A", T407="N"), J407="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O407" t="s">
@@ -39915,7 +39905,7 @@
         <v>44</v>
       </c>
       <c r="N408" t="str">
-        <f>IF(AND(OR(T408="A", T408="N"), J408="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O408" t="s">
@@ -39996,7 +39986,7 @@
         <v>44</v>
       </c>
       <c r="N409" t="str">
-        <f>IF(AND(OR(T409="A", T409="N"), J409="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O409" t="s">
@@ -40077,7 +40067,7 @@
         <v>44</v>
       </c>
       <c r="N410" t="str">
-        <f>IF(AND(OR(T410="A", T410="N"), J410="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O410" t="s">
@@ -40158,7 +40148,7 @@
         <v>43</v>
       </c>
       <c r="N411" t="str">
-        <f>IF(AND(OR(T411="A", T411="N"), J411="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O411" t="s">
@@ -40239,7 +40229,7 @@
         <v>44</v>
       </c>
       <c r="N412" t="str">
-        <f>IF(AND(OR(T412="A", T412="N"), J412="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O412" t="s">
@@ -40320,7 +40310,7 @@
         <v>44</v>
       </c>
       <c r="N413" t="str">
-        <f>IF(AND(OR(T413="A", T413="N"), J413="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O413" t="s">
@@ -40401,7 +40391,7 @@
         <v>44</v>
       </c>
       <c r="N414" t="str">
-        <f>IF(AND(OR(T414="A", T414="N"), J414="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O414" t="s">
@@ -40479,7 +40469,7 @@
         <v>44</v>
       </c>
       <c r="N415" t="str">
-        <f>IF(AND(OR(T415="A", T415="N"), J415="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O415" t="s">
@@ -40557,7 +40547,7 @@
         <v>44</v>
       </c>
       <c r="N416" t="str">
-        <f>IF(AND(OR(T416="A", T416="N"), J416="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O416" t="s">
@@ -40638,7 +40628,7 @@
         <v>44</v>
       </c>
       <c r="N417" t="str">
-        <f>IF(AND(OR(T417="A", T417="N"), J417="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O417" t="s">
@@ -40719,7 +40709,7 @@
         <v>44</v>
       </c>
       <c r="N418" t="str">
-        <f>IF(AND(OR(T418="A", T418="N"), J418="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O418" t="s">
@@ -40800,7 +40790,7 @@
         <v>43</v>
       </c>
       <c r="N419" t="str">
-        <f>IF(AND(OR(T419="A", T419="N"), J419="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O419" t="s">
@@ -40881,7 +40871,7 @@
         <v>44</v>
       </c>
       <c r="N420" t="str">
-        <f>IF(AND(OR(T420="A", T420="N"), J420="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O420" t="s">
@@ -40962,7 +40952,7 @@
         <v>44</v>
       </c>
       <c r="N421" t="str">
-        <f>IF(AND(OR(T421="A", T421="N"), J421="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O421" t="s">
@@ -41046,7 +41036,7 @@
         <v>44</v>
       </c>
       <c r="N422" t="str">
-        <f>IF(AND(OR(T422="A", T422="N"), J422="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O422" t="s">
@@ -41130,7 +41120,7 @@
         <v>43</v>
       </c>
       <c r="N423" t="str">
-        <f>IF(AND(OR(T423="A", T423="N"), J423="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O423" t="s">
@@ -41214,7 +41204,7 @@
         <v>44</v>
       </c>
       <c r="N424" t="str">
-        <f>IF(AND(OR(T424="A", T424="N"), J424="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O424" t="s">
@@ -41295,7 +41285,7 @@
         <v>44</v>
       </c>
       <c r="N425" t="str">
-        <f>IF(AND(OR(T425="A", T425="N"), J425="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O425" t="s">
@@ -41376,7 +41366,7 @@
         <v>43</v>
       </c>
       <c r="N426" t="str">
-        <f>IF(AND(OR(T426="A", T426="N"), J426="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O426" t="s">
@@ -41457,7 +41447,7 @@
         <v>44</v>
       </c>
       <c r="N427" t="str">
-        <f>IF(AND(OR(T427="A", T427="N"), J427="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O427" t="s">
@@ -41538,7 +41528,7 @@
         <v>44</v>
       </c>
       <c r="N428" t="str">
-        <f>IF(AND(OR(T428="A", T428="N"), J428="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O428" t="s">
@@ -41619,7 +41609,7 @@
         <v>44</v>
       </c>
       <c r="N429" t="str">
-        <f>IF(AND(OR(T429="A", T429="N"), J429="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O429" t="s">
@@ -41700,7 +41690,7 @@
         <v>44</v>
       </c>
       <c r="N430" t="str">
-        <f>IF(AND(OR(T430="A", T430="N"), J430="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O430" t="s">
@@ -41781,7 +41771,7 @@
         <v>44</v>
       </c>
       <c r="N431" t="str">
-        <f>IF(AND(OR(T431="A", T431="N"), J431="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O431" t="s">
@@ -41862,7 +41852,7 @@
         <v>44</v>
       </c>
       <c r="N432" t="str">
-        <f>IF(AND(OR(T432="A", T432="N"), J432="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O432" t="s">
@@ -41943,7 +41933,7 @@
         <v>44</v>
       </c>
       <c r="N433" t="str">
-        <f>IF(AND(OR(T433="A", T433="N"), J433="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O433" t="s">
@@ -42024,7 +42014,7 @@
         <v>44</v>
       </c>
       <c r="N434" t="str">
-        <f>IF(AND(OR(T434="A", T434="N"), J434="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O434" t="s">
@@ -42105,7 +42095,7 @@
         <v>44</v>
       </c>
       <c r="N435" t="str">
-        <f>IF(AND(OR(T435="A", T435="N"), J435="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O435" t="s">
@@ -42186,7 +42176,7 @@
         <v>44</v>
       </c>
       <c r="N436" t="str">
-        <f>IF(AND(OR(T436="A", T436="N"), J436="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O436" t="s">
@@ -42267,7 +42257,7 @@
         <v>43</v>
       </c>
       <c r="N437" t="str">
-        <f>IF(AND(OR(T437="A", T437="N"), J437="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O437" t="s">
@@ -42348,7 +42338,7 @@
         <v>44</v>
       </c>
       <c r="N438" t="str">
-        <f>IF(AND(OR(T438="A", T438="N"), J438="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O438" t="s">
@@ -42429,7 +42419,7 @@
         <v>44</v>
       </c>
       <c r="N439" t="str">
-        <f>IF(AND(OR(T439="A", T439="N"), J439="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O439" t="s">
@@ -42513,7 +42503,7 @@
         <v>44</v>
       </c>
       <c r="N440" t="str">
-        <f>IF(AND(OR(T440="A", T440="N"), J440="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O440" t="s">
@@ -42594,7 +42584,7 @@
         <v>44</v>
       </c>
       <c r="N441" t="str">
-        <f>IF(AND(OR(T441="A", T441="N"), J441="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O441" t="s">
@@ -42675,7 +42665,7 @@
         <v>43</v>
       </c>
       <c r="N442" t="str">
-        <f>IF(AND(OR(T442="A", T442="N"), J442="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O442" t="s">
@@ -42756,7 +42746,7 @@
         <v>43</v>
       </c>
       <c r="N443" t="str">
-        <f>IF(AND(OR(T443="A", T443="N"), J443="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O443" t="s">
@@ -42837,7 +42827,7 @@
         <v>44</v>
       </c>
       <c r="N444" t="str">
-        <f>IF(AND(OR(T444="A", T444="N"), J444="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O444" t="s">
@@ -42918,7 +42908,7 @@
         <v>43</v>
       </c>
       <c r="N445" t="str">
-        <f>IF(AND(OR(T445="A", T445="N"), J445="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O445" t="s">
@@ -42999,7 +42989,7 @@
         <v>44</v>
       </c>
       <c r="N446" t="str">
-        <f>IF(AND(OR(T446="A", T446="N"), J446="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O446" t="s">
@@ -43080,7 +43070,7 @@
         <v>44</v>
       </c>
       <c r="N447" t="str">
-        <f>IF(AND(OR(T447="A", T447="N"), J447="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O447" t="s">
@@ -43161,7 +43151,7 @@
         <v>43</v>
       </c>
       <c r="N448" t="str">
-        <f>IF(AND(OR(T448="A", T448="N"), J448="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O448" t="s">
@@ -43242,7 +43232,7 @@
         <v>44</v>
       </c>
       <c r="N449" t="str">
-        <f>IF(AND(OR(T449="A", T449="N"), J449="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="6"/>
         <v>Not Systemic</v>
       </c>
       <c r="O449" t="s">
@@ -43323,7 +43313,7 @@
         <v>44</v>
       </c>
       <c r="N450" t="str">
-        <f>IF(AND(OR(T450="A", T450="N"), J450="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" ref="N450:N509" si="7">IF(AND(OR(T450="A", T450="N"), J450="Yes"), "Potentially Systemic", "Not Systemic")</f>
         <v>Not Systemic</v>
       </c>
       <c r="O450" t="s">
@@ -43407,7 +43397,7 @@
         <v>43</v>
       </c>
       <c r="N451" t="str">
-        <f>IF(AND(OR(T451="A", T451="N"), J451="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O451" t="s">
@@ -43491,7 +43481,7 @@
         <v>44</v>
       </c>
       <c r="N452" t="str">
-        <f>IF(AND(OR(T452="A", T452="N"), J452="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O452" t="s">
@@ -43572,7 +43562,7 @@
         <v>44</v>
       </c>
       <c r="N453" t="str">
-        <f>IF(AND(OR(T453="A", T453="N"), J453="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O453" t="s">
@@ -43653,7 +43643,7 @@
         <v>44</v>
       </c>
       <c r="N454" t="str">
-        <f>IF(AND(OR(T454="A", T454="N"), J454="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O454" t="s">
@@ -43734,7 +43724,7 @@
         <v>44</v>
       </c>
       <c r="N455" t="str">
-        <f>IF(AND(OR(T455="A", T455="N"), J455="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O455" t="s">
@@ -43815,7 +43805,7 @@
         <v>44</v>
       </c>
       <c r="N456" t="str">
-        <f>IF(AND(OR(T456="A", T456="N"), J456="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O456" t="s">
@@ -43896,7 +43886,7 @@
         <v>43</v>
       </c>
       <c r="N457" t="str">
-        <f>IF(AND(OR(T457="A", T457="N"), J457="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O457" t="s">
@@ -43977,7 +43967,7 @@
         <v>44</v>
       </c>
       <c r="N458" t="str">
-        <f>IF(AND(OR(T458="A", T458="N"), J458="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O458" t="s">
@@ -44058,7 +44048,7 @@
         <v>44</v>
       </c>
       <c r="N459" t="str">
-        <f>IF(AND(OR(T459="A", T459="N"), J459="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O459" t="s">
@@ -44139,7 +44129,7 @@
         <v>43</v>
       </c>
       <c r="N460" t="str">
-        <f>IF(AND(OR(T460="A", T460="N"), J460="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O460" t="s">
@@ -44220,7 +44210,7 @@
         <v>44</v>
       </c>
       <c r="N461" t="str">
-        <f>IF(AND(OR(T461="A", T461="N"), J461="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O461" t="s">
@@ -44301,7 +44291,7 @@
         <v>44</v>
       </c>
       <c r="N462" t="str">
-        <f>IF(AND(OR(T462="A", T462="N"), J462="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O462" t="s">
@@ -44382,7 +44372,7 @@
         <v>44</v>
       </c>
       <c r="N463" t="str">
-        <f>IF(AND(OR(T463="A", T463="N"), J463="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O463" t="s">
@@ -44463,7 +44453,7 @@
         <v>43</v>
       </c>
       <c r="N464" t="str">
-        <f>IF(AND(OR(T464="A", T464="N"), J464="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O464" t="s">
@@ -44544,7 +44534,7 @@
         <v>44</v>
       </c>
       <c r="N465" t="str">
-        <f>IF(AND(OR(T465="A", T465="N"), J465="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O465" t="s">
@@ -44625,7 +44615,7 @@
         <v>44</v>
       </c>
       <c r="N466" t="str">
-        <f>IF(AND(OR(T466="A", T466="N"), J466="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O466" t="s">
@@ -44706,7 +44696,7 @@
         <v>43</v>
       </c>
       <c r="N467" t="str">
-        <f>IF(AND(OR(T467="A", T467="N"), J467="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O467" t="s">
@@ -44787,7 +44777,7 @@
         <v>44</v>
       </c>
       <c r="N468" t="str">
-        <f>IF(AND(OR(T468="A", T468="N"), J468="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O468" t="s">
@@ -44868,7 +44858,7 @@
         <v>43</v>
       </c>
       <c r="N469" t="str">
-        <f>IF(AND(OR(T469="A", T469="N"), J469="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O469" t="s">
@@ -44949,7 +44939,7 @@
         <v>44</v>
       </c>
       <c r="N470" t="str">
-        <f>IF(AND(OR(T470="A", T470="N"), J470="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O470" t="s">
@@ -45030,7 +45020,7 @@
         <v>44</v>
       </c>
       <c r="N471" t="str">
-        <f>IF(AND(OR(T471="A", T471="N"), J471="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O471" t="s">
@@ -45111,7 +45101,7 @@
         <v>44</v>
       </c>
       <c r="N472" t="str">
-        <f>IF(AND(OR(T472="A", T472="N"), J472="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O472" t="s">
@@ -45192,7 +45182,7 @@
         <v>44</v>
       </c>
       <c r="N473" t="str">
-        <f>IF(AND(OR(T473="A", T473="N"), J473="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O473" t="s">
@@ -45273,7 +45263,7 @@
         <v>44</v>
       </c>
       <c r="N474" t="str">
-        <f>IF(AND(OR(T474="A", T474="N"), J474="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O474" t="s">
@@ -45354,7 +45344,7 @@
         <v>44</v>
       </c>
       <c r="N475" t="str">
-        <f>IF(AND(OR(T475="A", T475="N"), J475="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O475" t="s">
@@ -45432,7 +45422,7 @@
         <v>44</v>
       </c>
       <c r="N476" t="str">
-        <f>IF(AND(OR(T476="A", T476="N"), J476="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O476" t="s">
@@ -45513,7 +45503,7 @@
         <v>43</v>
       </c>
       <c r="N477" t="str">
-        <f>IF(AND(OR(T477="A", T477="N"), J477="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O477" t="s">
@@ -45594,7 +45584,7 @@
         <v>44</v>
       </c>
       <c r="N478" t="str">
-        <f>IF(AND(OR(T478="A", T478="N"), J478="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O478" t="s">
@@ -45675,7 +45665,7 @@
         <v>43</v>
       </c>
       <c r="N479" t="str">
-        <f>IF(AND(OR(T479="A", T479="N"), J479="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O479" t="s">
@@ -45756,7 +45746,7 @@
         <v>43</v>
       </c>
       <c r="N480" t="str">
-        <f>IF(AND(OR(T480="A", T480="N"), J480="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O480" t="s">
@@ -45837,7 +45827,7 @@
         <v>44</v>
       </c>
       <c r="N481" t="str">
-        <f>IF(AND(OR(T481="A", T481="N"), J481="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O481" t="s">
@@ -45918,7 +45908,7 @@
         <v>44</v>
       </c>
       <c r="N482" t="str">
-        <f>IF(AND(OR(T482="A", T482="N"), J482="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O482" t="s">
@@ -45999,7 +45989,7 @@
         <v>44</v>
       </c>
       <c r="N483" t="str">
-        <f>IF(AND(OR(T483="A", T483="N"), J483="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O483" t="s">
@@ -46080,7 +46070,7 @@
         <v>44</v>
       </c>
       <c r="N484" t="str">
-        <f>IF(AND(OR(T484="A", T484="N"), J484="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O484" t="s">
@@ -46161,7 +46151,7 @@
         <v>44</v>
       </c>
       <c r="N485" t="str">
-        <f>IF(AND(OR(T485="A", T485="N"), J485="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O485" t="s">
@@ -46242,7 +46232,7 @@
         <v>44</v>
       </c>
       <c r="N486" t="str">
-        <f>IF(AND(OR(T486="A", T486="N"), J486="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O486" t="s">
@@ -46323,7 +46313,7 @@
         <v>44</v>
       </c>
       <c r="N487" t="str">
-        <f>IF(AND(OR(T487="A", T487="N"), J487="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O487" t="s">
@@ -46404,7 +46394,7 @@
         <v>44</v>
       </c>
       <c r="N488" t="str">
-        <f>IF(AND(OR(T488="A", T488="N"), J488="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O488" t="s">
@@ -46485,7 +46475,7 @@
         <v>44</v>
       </c>
       <c r="N489" t="str">
-        <f>IF(AND(OR(T489="A", T489="N"), J489="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O489" t="s">
@@ -46566,7 +46556,7 @@
         <v>43</v>
       </c>
       <c r="N490" t="str">
-        <f>IF(AND(OR(T490="A", T490="N"), J490="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O490" t="s">
@@ -46647,7 +46637,7 @@
         <v>44</v>
       </c>
       <c r="N491" t="str">
-        <f>IF(AND(OR(T491="A", T491="N"), J491="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O491" t="s">
@@ -46728,7 +46718,7 @@
         <v>44</v>
       </c>
       <c r="N492" t="str">
-        <f>IF(AND(OR(T492="A", T492="N"), J492="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O492" t="s">
@@ -46809,7 +46799,7 @@
         <v>43</v>
       </c>
       <c r="N493" t="str">
-        <f>IF(AND(OR(T493="A", T493="N"), J493="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O493" t="s">
@@ -46890,7 +46880,7 @@
         <v>44</v>
       </c>
       <c r="N494" t="str">
-        <f>IF(AND(OR(T494="A", T494="N"), J494="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O494" t="s">
@@ -46971,7 +46961,7 @@
         <v>44</v>
       </c>
       <c r="N495" t="str">
-        <f>IF(AND(OR(T495="A", T495="N"), J495="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O495" t="s">
@@ -47052,7 +47042,7 @@
         <v>44</v>
       </c>
       <c r="N496" t="str">
-        <f>IF(AND(OR(T496="A", T496="N"), J496="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O496" t="s">
@@ -47133,7 +47123,7 @@
         <v>44</v>
       </c>
       <c r="N497" t="str">
-        <f>IF(AND(OR(T497="A", T497="N"), J497="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O497" t="s">
@@ -47214,7 +47204,7 @@
         <v>43</v>
       </c>
       <c r="N498" t="str">
-        <f>IF(AND(OR(T498="A", T498="N"), J498="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O498" t="s">
@@ -47295,7 +47285,7 @@
         <v>43</v>
       </c>
       <c r="N499" t="str">
-        <f>IF(AND(OR(T499="A", T499="N"), J499="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O499" t="s">
@@ -47376,7 +47366,7 @@
         <v>44</v>
       </c>
       <c r="N500" t="str">
-        <f>IF(AND(OR(T500="A", T500="N"), J500="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O500" t="s">
@@ -47457,7 +47447,7 @@
         <v>44</v>
       </c>
       <c r="N501" t="str">
-        <f>IF(AND(OR(T501="A", T501="N"), J501="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O501" t="s">
@@ -47538,7 +47528,7 @@
         <v>43</v>
       </c>
       <c r="N502" t="str">
-        <f>IF(AND(OR(T502="A", T502="N"), J502="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O502" t="s">
@@ -47619,7 +47609,7 @@
         <v>43</v>
       </c>
       <c r="N503" t="str">
-        <f>IF(AND(OR(T503="A", T503="N"), J503="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O503" t="s">
@@ -47700,7 +47690,7 @@
         <v>44</v>
       </c>
       <c r="N504" t="str">
-        <f>IF(AND(OR(T504="A", T504="N"), J504="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O504" t="s">
@@ -47781,7 +47771,7 @@
         <v>43</v>
       </c>
       <c r="N505" t="str">
-        <f>IF(AND(OR(T505="A", T505="N"), J505="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O505" t="s">
@@ -47862,7 +47852,7 @@
         <v>43</v>
       </c>
       <c r="N506" t="str">
-        <f>IF(AND(OR(T506="A", T506="N"), J506="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O506" t="s">
@@ -47943,7 +47933,7 @@
         <v>43</v>
       </c>
       <c r="N507" t="str">
-        <f>IF(AND(OR(T507="A", T507="N"), J507="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Potentially Systemic</v>
       </c>
       <c r="O507" t="s">
@@ -48024,7 +48014,7 @@
         <v>43</v>
       </c>
       <c r="N508" t="str">
-        <f>IF(AND(OR(T508="A", T508="N"), J508="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O508" t="s">
@@ -48096,7 +48086,7 @@
         <v>43</v>
       </c>
       <c r="N509" t="str">
-        <f>IF(AND(OR(T509="A", T509="N"), J509="Yes"), "Potentially Systemic", "Not Systemic")</f>
+        <f t="shared" si="7"/>
         <v>Not Systemic</v>
       </c>
       <c r="O509" t="s">
@@ -48140,7 +48130,6 @@
       </c>
     </row>
     <row r="510" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A510" s="2"/>
       <c r="N510">
         <f>SUBTOTAL(103,Table2[Systemic])</f>
         <v>508</v>

</xml_diff>